<commit_message>
MR24-045 D10 (no titer data)
</commit_message>
<xml_diff>
--- a/data/mr24-045-experiment/MR24-045-MasterDataTable.xlsx
+++ b/data/mr24-045-experiment/MR24-045-MasterDataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/MR24-045-MPC-3L/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1470" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{970C3D87-E5E3-4C81-A6EA-E66F76EC7286}"/>
+  <xr:revisionPtr revIDLastSave="1540" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A3C3CC1-DA82-4F96-AE15-07BC88948B97}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="90">
   <si>
     <t>Batch Data</t>
   </si>
@@ -307,6 +307,9 @@
   <si>
     <t>MR24-045-806</t>
   </si>
+  <si>
+    <t>Antifoam totalizer reset due to schedule restart</t>
+  </si>
 </sst>
 </file>
 
@@ -318,7 +321,7 @@
     <numFmt numFmtId="166" formatCode="0.00000"/>
     <numFmt numFmtId="167" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,6 +513,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -990,7 +1000,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1134,6 +1144,9 @@
     <xf numFmtId="0" fontId="19" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1229,6 +1242,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9172,7 +9189,7 @@
         <v>84.700000000000045</v>
       </c>
       <c r="AS35" s="45">
-        <f t="shared" ref="AS35:AS66" si="60">AQ35-AR35</f>
+        <f t="shared" ref="AS35:AS65" si="60">AQ35-AR35</f>
         <v>1755.3</v>
       </c>
       <c r="AT35" s="45">
@@ -12650,7 +12667,9 @@
       <c r="D51" s="3">
         <v>8</v>
       </c>
-      <c r="E51" s="3"/>
+      <c r="E51" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="F51" s="60">
         <v>45541.409976851901</v>
       </c>
@@ -12744,7 +12763,7 @@
       <c r="AK51" s="44">
         <v>33.090000000000003</v>
       </c>
-      <c r="AL51" s="6">
+      <c r="AL51" s="87">
         <v>5.29</v>
       </c>
       <c r="AM51" s="42">
@@ -12877,6 +12896,9 @@
       <c r="D52">
         <v>8</v>
       </c>
+      <c r="E52" t="s">
+        <v>89</v>
+      </c>
       <c r="F52" s="61">
         <v>45541.414027777799</v>
       </c>
@@ -12970,7 +12992,7 @@
       <c r="AK52" s="44">
         <v>26.68</v>
       </c>
-      <c r="AL52" s="44">
+      <c r="AL52" s="88">
         <v>3</v>
       </c>
       <c r="AM52" s="45">
@@ -13103,6 +13125,9 @@
       <c r="D53">
         <v>8</v>
       </c>
+      <c r="E53" t="s">
+        <v>89</v>
+      </c>
       <c r="F53" s="61">
         <v>45541.418136574102</v>
       </c>
@@ -13196,7 +13221,7 @@
       <c r="AK53" s="44">
         <v>1.24</v>
       </c>
-      <c r="AL53" s="44">
+      <c r="AL53" s="88">
         <v>6.66</v>
       </c>
       <c r="AM53" s="45">
@@ -13329,6 +13354,9 @@
       <c r="D54">
         <v>8</v>
       </c>
+      <c r="E54" t="s">
+        <v>89</v>
+      </c>
       <c r="F54" s="61">
         <v>45541.4217361111</v>
       </c>
@@ -13420,7 +13448,7 @@
       <c r="AK54" s="44">
         <v>10.53</v>
       </c>
-      <c r="AL54" s="44">
+      <c r="AL54" s="88">
         <v>6.76</v>
       </c>
       <c r="AM54" s="45">
@@ -13550,6 +13578,9 @@
       <c r="D55">
         <v>8</v>
       </c>
+      <c r="E55" t="s">
+        <v>89</v>
+      </c>
       <c r="F55" s="61">
         <v>45541.425601851901</v>
       </c>
@@ -13641,7 +13672,7 @@
       <c r="AK55" s="44">
         <v>7.31</v>
       </c>
-      <c r="AL55" s="44">
+      <c r="AL55" s="88">
         <v>6.44</v>
       </c>
       <c r="AM55" s="45">
@@ -13771,7 +13802,9 @@
       <c r="D56" s="5">
         <v>8</v>
       </c>
-      <c r="E56" s="5"/>
+      <c r="E56" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="F56" s="62">
         <v>45541.429097222201</v>
       </c>
@@ -13865,7 +13898,7 @@
       <c r="AK56" s="7">
         <v>28.23</v>
       </c>
-      <c r="AL56" s="7">
+      <c r="AL56" s="89">
         <v>6.52</v>
       </c>
       <c r="AM56" s="41">
@@ -13997,7 +14030,9 @@
         <v>9</v>
       </c>
       <c r="E57" s="3"/>
-      <c r="F57" s="60"/>
+      <c r="F57" s="60">
+        <v>45542.536215277803</v>
+      </c>
       <c r="G57" s="3">
         <v>4805.7299999999996</v>
       </c>
@@ -14094,7 +14129,7 @@
       </c>
       <c r="AM57" s="42">
         <f>BR57</f>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="AN57" s="6">
         <v>150.99</v>
@@ -14146,8 +14181,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC57" s="8"/>
-      <c r="BD57" s="9"/>
-      <c r="BE57" s="21"/>
+      <c r="BD57" s="46">
+        <f>BM57*24*60/BH57</f>
+        <v>1.2227344977136538E-2</v>
+      </c>
+      <c r="BE57" s="22">
+        <f>BP57/BH57</f>
+        <v>9.9999999999999995E-8</v>
+      </c>
       <c r="BF57" s="8">
         <f t="shared" si="17"/>
         <v>1.1345033880000001E-2</v>
@@ -14170,15 +14211,14 @@
       </c>
       <c r="BK57" s="10">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>22.446544179298034</v>
       </c>
       <c r="BL57" s="10" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM57" s="10">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="BN57" s="35" t="str">
         <f t="shared" si="32"/>
@@ -14189,20 +14229,19 @@
         <v/>
       </c>
       <c r="BP57" s="50">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>1.8357660000000001E-4</v>
       </c>
       <c r="BQ57" s="27">
         <f>IF(BL57&lt;&gt;"",BL57/0.000385,IF(BM57&lt;&gt;"",BM57/0.000385,BN57/0.000385))</f>
-        <v>0</v>
+        <v>40.487994551403375</v>
       </c>
       <c r="BR57" s="37">
         <f>IF(BL57&lt;&gt;"",BL57,IF(BM57&lt;&gt;"",BM57,BN57))</f>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="BS57" s="32">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>1.8357660000000001E-4</v>
       </c>
     </row>
     <row r="58" spans="1:71" x14ac:dyDescent="0.3">
@@ -14218,7 +14257,9 @@
       <c r="D58">
         <v>9</v>
       </c>
-      <c r="F58" s="61"/>
+      <c r="F58" s="61">
+        <v>45542.542280092603</v>
+      </c>
       <c r="G58">
         <v>4805.7299999999996</v>
       </c>
@@ -14315,7 +14356,7 @@
       </c>
       <c r="AM58" s="45">
         <f t="shared" ref="AM58:AM62" si="75">BR58</f>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="AN58" s="44">
         <v>167.56</v>
@@ -14367,8 +14408,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC58" s="11"/>
-      <c r="BD58" s="46"/>
-      <c r="BE58" s="22"/>
+      <c r="BD58" s="46">
+        <f>BM58*24*60/BH58</f>
+        <v>1.1176787745194918E-2</v>
+      </c>
+      <c r="BE58" s="22">
+        <f>BP58/BH58</f>
+        <v>3.3316909083529549E-3</v>
+      </c>
       <c r="BF58" s="11">
         <f t="shared" si="17"/>
         <v>1.1502565799999998E-2</v>
@@ -14391,15 +14438,14 @@
       </c>
       <c r="BK58" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>20.504264190069886</v>
       </c>
       <c r="BL58" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM58" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="BN58" s="48" t="str">
         <f t="shared" si="32"/>
@@ -14410,20 +14456,19 @@
         <v/>
       </c>
       <c r="BP58" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>6.1121202390098297</v>
       </c>
       <c r="BQ58" s="28">
         <f t="shared" ref="BQ58:BQ62" si="76">IF(BL58&lt;&gt;"",BL58/0.000385,IF(BM58&lt;&gt;"",BM58/0.000385,BN58/0.000385))</f>
-        <v>0</v>
+        <v>36.984603517442082</v>
       </c>
       <c r="BR58" s="49">
         <f t="shared" ref="BR58:BR62" si="77">IF(BL58&lt;&gt;"",BL58,IF(BM58&lt;&gt;"",BM58,BN58))</f>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="BS58" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>6.1121202390098297</v>
       </c>
     </row>
     <row r="59" spans="1:71" x14ac:dyDescent="0.3">
@@ -14439,7 +14484,9 @@
       <c r="D59">
         <v>9</v>
       </c>
-      <c r="F59" s="61"/>
+      <c r="F59" s="61">
+        <v>45542.544826388897</v>
+      </c>
       <c r="G59">
         <v>4805.7299999999996</v>
       </c>
@@ -14536,7 +14583,7 @@
       </c>
       <c r="AM59" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="AN59" s="44">
         <v>211.31</v>
@@ -14588,8 +14635,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC59" s="11"/>
-      <c r="BD59" s="46"/>
-      <c r="BE59" s="22"/>
+      <c r="BD59" s="46">
+        <f>BM59*24*60/BH59</f>
+        <v>2.3999999999999973E-2</v>
+      </c>
+      <c r="BE59" s="22">
+        <f>BP59/BH59</f>
+        <v>4.1250564909925723E-3</v>
+      </c>
       <c r="BF59" s="11">
         <f t="shared" si="17"/>
         <v>9.8997816750000002E-3</v>
@@ -14612,15 +14665,14 @@
       </c>
       <c r="BK59" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>45.256144799999952</v>
       </c>
       <c r="BL59" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM59" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="BN59" s="48" t="str">
         <f t="shared" si="32"/>
@@ -14631,20 +14683,19 @@
         <v/>
       </c>
       <c r="BP59" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>7.77850641102249</v>
       </c>
       <c r="BQ59" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>81.630852813852727</v>
       </c>
       <c r="BR59" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="BS59" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>7.77850641102249</v>
       </c>
     </row>
     <row r="60" spans="1:71" x14ac:dyDescent="0.3">
@@ -14660,13 +14711,15 @@
       <c r="D60">
         <v>9</v>
       </c>
-      <c r="F60" s="61"/>
+      <c r="F60" s="61">
+        <v>45542.547604166699</v>
+      </c>
       <c r="G60">
         <v>4805.7299999999996</v>
       </c>
       <c r="H60" s="44"/>
       <c r="I60" s="44">
-        <v>4576.09</v>
+        <v>4576.0950000000003</v>
       </c>
       <c r="J60" s="44">
         <v>19.2</v>
@@ -14757,7 +14810,7 @@
       </c>
       <c r="AM60" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="AN60" s="44">
         <v>204.07</v>
@@ -14808,7 +14861,9 @@
       <c r="BB60" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC60" s="11"/>
+      <c r="BC60" s="11">
+        <v>1.7999999999999999E-2</v>
+      </c>
       <c r="BE60" s="22"/>
       <c r="BF60" s="11">
         <f t="shared" si="17"/>
@@ -14832,11 +14887,11 @@
       </c>
       <c r="BK60" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>33.966593999999986</v>
       </c>
       <c r="BL60" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="BM60" s="48" t="str">
         <f t="shared" si="31"/>
@@ -14856,11 +14911,11 @@
       </c>
       <c r="BQ60" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>61.267305194805189</v>
       </c>
       <c r="BR60" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="BS60" s="30">
         <f t="shared" si="21"/>
@@ -14880,7 +14935,9 @@
       <c r="D61">
         <v>9</v>
       </c>
-      <c r="F61" s="61"/>
+      <c r="F61" s="61">
+        <v>45542.550289351901</v>
+      </c>
       <c r="G61">
         <v>4805.7299999999996</v>
       </c>
@@ -14975,7 +15032,7 @@
       </c>
       <c r="AM61" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="AN61" s="44">
         <v>227.05</v>
@@ -15026,7 +15083,9 @@
       <c r="BB61" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC61" s="11"/>
+      <c r="BC61" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BE61" s="22"/>
       <c r="BF61" s="11">
         <f t="shared" si="17"/>
@@ -15050,11 +15109,11 @@
       </c>
       <c r="BK61" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>39.638652000000008</v>
       </c>
       <c r="BL61" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="BM61" s="48" t="str">
         <f t="shared" si="31"/>
@@ -15074,11 +15133,11 @@
       </c>
       <c r="BQ61" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>71.498290043290055</v>
       </c>
       <c r="BR61" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="BS61" s="30">
         <f t="shared" si="21"/>
@@ -15099,7 +15158,9 @@
         <v>9</v>
       </c>
       <c r="E62" s="5"/>
-      <c r="F62" s="62"/>
+      <c r="F62" s="62">
+        <v>45542.552824074097</v>
+      </c>
       <c r="G62" s="5">
         <v>4805.7299999999996</v>
       </c>
@@ -15196,7 +15257,7 @@
       </c>
       <c r="AM62" s="41">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="AN62" s="7">
         <v>187.96</v>
@@ -15247,7 +15308,9 @@
       <c r="BB62" s="23">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC62" s="12"/>
+      <c r="BC62" s="12">
+        <v>8.5000000000000006E-3</v>
+      </c>
       <c r="BD62" s="5"/>
       <c r="BE62" s="23"/>
       <c r="BF62" s="12">
@@ -15272,11 +15335,11 @@
       </c>
       <c r="BK62" s="14">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>15.886534000000001</v>
       </c>
       <c r="BL62" s="14">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="BM62" s="48" t="str">
         <f t="shared" si="31"/>
@@ -15296,11 +15359,11 @@
       </c>
       <c r="BQ62" s="29">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>28.655364357864364</v>
       </c>
       <c r="BR62" s="38">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="BS62" s="31">
         <f t="shared" si="21"/>
@@ -15321,70 +15384,135 @@
         <v>10</v>
       </c>
       <c r="E63" s="3"/>
-      <c r="F63" s="60"/>
+      <c r="F63" s="60">
+        <v>45543.405208333301</v>
+      </c>
       <c r="G63" s="63">
         <v>5497.99</v>
       </c>
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
-      <c r="J63" s="6"/>
-      <c r="K63" s="6"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="6"/>
-      <c r="N63" s="6"/>
-      <c r="O63" s="6"/>
-      <c r="P63" s="6"/>
-      <c r="Q63" s="6"/>
+      <c r="J63" s="6">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="K63" s="6">
+        <v>18.7</v>
+      </c>
+      <c r="L63" s="6">
+        <v>91.5</v>
+      </c>
+      <c r="M63" s="6">
+        <v>17.3</v>
+      </c>
+      <c r="N63" s="6">
+        <v>347</v>
+      </c>
+      <c r="O63" s="6">
+        <v>1.72</v>
+      </c>
+      <c r="P63" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="Q63" s="6">
+        <v>1.64</v>
+      </c>
       <c r="R63" s="6"/>
-      <c r="S63" s="6"/>
-      <c r="T63" s="6"/>
-      <c r="U63" s="6"/>
-      <c r="V63" s="6"/>
-      <c r="W63" s="6"/>
-      <c r="X63" s="6"/>
-      <c r="Y63" s="6"/>
-      <c r="Z63" s="6"/>
-      <c r="AA63" s="6"/>
-      <c r="AB63" s="6"/>
-      <c r="AC63" s="6"/>
-      <c r="AD63" s="16"/>
-      <c r="AE63" s="6"/>
-      <c r="AF63" s="6"/>
-      <c r="AG63" s="6"/>
+      <c r="S63" s="6">
+        <v>0.11</v>
+      </c>
+      <c r="T63" s="6">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="U63" s="6">
+        <v>0.16</v>
+      </c>
+      <c r="V63" s="6">
+        <v>7.2460000000000004</v>
+      </c>
+      <c r="W63" s="6">
+        <v>95.9</v>
+      </c>
+      <c r="X63" s="6">
+        <v>11.5</v>
+      </c>
+      <c r="Y63" s="6">
+        <v>2.23</v>
+      </c>
+      <c r="Z63" s="6">
+        <v>146.4</v>
+      </c>
+      <c r="AA63" s="6">
+        <v>40.6</v>
+      </c>
+      <c r="AB63" s="6">
+        <v>84.1</v>
+      </c>
+      <c r="AC63" s="6">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="AD63" s="16">
+        <v>7.2869999999999999</v>
+      </c>
+      <c r="AE63" s="6">
+        <v>300</v>
+      </c>
+      <c r="AF63" s="6">
+        <v>47.8</v>
+      </c>
+      <c r="AG63" s="6">
+        <v>7.29</v>
+      </c>
       <c r="AH63" s="40">
         <f>AF63/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI63" s="6"/>
-      <c r="AJ63" s="6"/>
-      <c r="AK63" s="44"/>
-      <c r="AL63" s="6"/>
+        <v>0.47799999999999998</v>
+      </c>
+      <c r="AI63" s="6">
+        <v>34</v>
+      </c>
+      <c r="AJ63" s="6">
+        <v>22.065000000000001</v>
+      </c>
+      <c r="AK63" s="44">
+        <v>44.018999999999998</v>
+      </c>
+      <c r="AL63" s="6">
+        <f>AL51+1.91</f>
+        <v>7.2</v>
+      </c>
       <c r="AM63" s="42">
         <f>BR63</f>
-        <v>0</v>
-      </c>
-      <c r="AN63" s="6"/>
-      <c r="AO63" s="6"/>
-      <c r="AP63" s="6"/>
-      <c r="AQ63" s="6"/>
+        <v>5.1207888888888803E-3</v>
+      </c>
+      <c r="AN63" s="6">
+        <v>169.89</v>
+      </c>
+      <c r="AO63" s="6">
+        <v>65.31</v>
+      </c>
+      <c r="AP63" s="6">
+        <v>497</v>
+      </c>
+      <c r="AQ63" s="6">
+        <v>1984</v>
+      </c>
       <c r="AR63" s="40">
         <v>137.11999999999989</v>
       </c>
       <c r="AS63" s="40">
         <f t="shared" si="60"/>
-        <v>-137.11999999999989</v>
+        <v>1846.88</v>
       </c>
       <c r="AT63" s="40">
         <f t="shared" si="36"/>
-        <v>-150.99</v>
+        <v>18.899999999999977</v>
       </c>
       <c r="AU63" s="40">
         <f t="shared" si="37"/>
-        <v>-65.31</v>
+        <v>0</v>
       </c>
       <c r="AV63" s="40">
         <f t="shared" si="65"/>
-        <v>518</v>
+        <v>21</v>
       </c>
       <c r="AW63" s="24">
         <v>15</v>
@@ -15405,39 +15533,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC63" s="8"/>
-      <c r="BD63" s="9"/>
-      <c r="BE63" s="21"/>
+      <c r="BD63" s="46">
+        <f>BM63*24*60/BH63</f>
+        <v>3.999999999999994E-3</v>
+      </c>
+      <c r="BE63" s="22">
+        <f>BP63/BH63</f>
+        <v>3.9797979551218672E-3</v>
+      </c>
       <c r="BF63" s="8">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.0341945239999999E-2</v>
       </c>
       <c r="BG63" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.892401145599999</v>
       </c>
       <c r="BH63" s="9">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI63" s="10" t="str">
+        <v>1843.4839999999999</v>
+      </c>
+      <c r="BI63" s="10">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ63" s="10" t="str">
+        <v>9.2157024416810771E-2</v>
+      </c>
+      <c r="BJ63" s="10">
         <f t="shared" si="9"/>
-        <v/>
+        <v>9.9935294117647053E-2</v>
       </c>
       <c r="BK63" s="10">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>7.3739359999999881</v>
       </c>
       <c r="BL63" s="10" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM63" s="10">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>5.1207888888888803E-3</v>
       </c>
       <c r="BN63" s="35" t="str">
         <f t="shared" si="32"/>
@@ -15448,20 +15581,19 @@
         <v/>
       </c>
       <c r="BP63" s="50">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>7.33669385349988</v>
       </c>
       <c r="BQ63" s="27">
         <f>IF(BL63&lt;&gt;"",BL63/0.000385,IF(BM63&lt;&gt;"",BM63/0.000385,BN63/0.000385))</f>
-        <v>0</v>
+        <v>13.300750360750339</v>
       </c>
       <c r="BR63" s="37">
         <f>IF(BL63&lt;&gt;"",BL63,IF(BM63&lt;&gt;"",BM63,BN63))</f>
-        <v>0</v>
+        <v>5.1207888888888803E-3</v>
       </c>
       <c r="BS63" s="32">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>7.33669385349988</v>
       </c>
     </row>
     <row r="64" spans="1:71" x14ac:dyDescent="0.3">
@@ -15477,70 +15609,135 @@
       <c r="D64">
         <v>10</v>
       </c>
-      <c r="F64" s="61"/>
+      <c r="F64" s="61">
+        <v>45543.413275462997</v>
+      </c>
       <c r="G64" s="64">
         <v>5497.99</v>
       </c>
       <c r="H64" s="44"/>
       <c r="I64" s="44"/>
-      <c r="J64" s="44"/>
-      <c r="K64" s="44"/>
-      <c r="L64" s="44"/>
-      <c r="M64" s="44"/>
-      <c r="N64" s="44"/>
-      <c r="O64" s="44"/>
-      <c r="P64" s="44"/>
-      <c r="Q64" s="44"/>
+      <c r="J64" s="44">
+        <v>20.6</v>
+      </c>
+      <c r="K64" s="44">
+        <v>19.3</v>
+      </c>
+      <c r="L64" s="44">
+        <v>93.9</v>
+      </c>
+      <c r="M64" s="44">
+        <v>17.8</v>
+      </c>
+      <c r="N64" s="44">
+        <v>348</v>
+      </c>
+      <c r="O64" s="44">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="P64" s="44">
+        <v>0.21</v>
+      </c>
+      <c r="Q64" s="44">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="R64" s="44"/>
-      <c r="S64" s="44"/>
-      <c r="T64" s="44"/>
-      <c r="U64" s="44"/>
-      <c r="V64" s="44"/>
-      <c r="W64" s="44"/>
-      <c r="X64" s="44"/>
-      <c r="Y64" s="44"/>
-      <c r="Z64" s="44"/>
-      <c r="AA64" s="44"/>
-      <c r="AB64" s="44"/>
-      <c r="AC64" s="44"/>
-      <c r="AD64" s="17"/>
-      <c r="AE64" s="44"/>
-      <c r="AF64" s="44"/>
-      <c r="AG64" s="44"/>
+      <c r="S64" s="44">
+        <v>0.1</v>
+      </c>
+      <c r="T64" s="44">
+        <v>0.15</v>
+      </c>
+      <c r="U64" s="44">
+        <v>0.16</v>
+      </c>
+      <c r="V64" s="44">
+        <v>7.2619999999999996</v>
+      </c>
+      <c r="W64" s="44">
+        <v>105</v>
+      </c>
+      <c r="X64" s="44">
+        <v>55.7</v>
+      </c>
+      <c r="Y64" s="44">
+        <v>2.15</v>
+      </c>
+      <c r="Z64" s="44">
+        <v>154.19999999999999</v>
+      </c>
+      <c r="AA64" s="44">
+        <v>46.1</v>
+      </c>
+      <c r="AB64" s="44">
+        <v>92.1</v>
+      </c>
+      <c r="AC64" s="44">
+        <v>45.2</v>
+      </c>
+      <c r="AD64" s="17">
+        <v>7.3029999999999999</v>
+      </c>
+      <c r="AE64" s="44">
+        <v>300</v>
+      </c>
+      <c r="AF64" s="44">
+        <v>49.9</v>
+      </c>
+      <c r="AG64" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH64" s="45">
         <f t="shared" ref="AH64:AH68" si="78">AF64/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI64" s="44"/>
-      <c r="AJ64" s="44"/>
-      <c r="AK64" s="44"/>
-      <c r="AL64" s="44"/>
+        <v>0.499</v>
+      </c>
+      <c r="AI64" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ64" s="44">
+        <v>24.568000000000001</v>
+      </c>
+      <c r="AK64" s="44">
+        <v>27.469000000000001</v>
+      </c>
+      <c r="AL64" s="44">
+        <f>AL52+1.86</f>
+        <v>4.8600000000000003</v>
+      </c>
       <c r="AM64" s="45">
         <f t="shared" ref="AM64:AM68" si="79">BR64</f>
-        <v>0</v>
-      </c>
-      <c r="AN64" s="44"/>
-      <c r="AO64" s="44"/>
-      <c r="AP64" s="44"/>
-      <c r="AQ64" s="44"/>
+        <v>1.1401776999282799E-2</v>
+      </c>
+      <c r="AN64" s="44">
+        <v>185.31</v>
+      </c>
+      <c r="AO64" s="44">
+        <v>68.25</v>
+      </c>
+      <c r="AP64" s="44">
+        <v>481</v>
+      </c>
+      <c r="AQ64" s="44">
+        <v>1988</v>
+      </c>
       <c r="AR64" s="45">
         <v>45.769999999999982</v>
       </c>
       <c r="AS64" s="45">
         <f t="shared" si="60"/>
-        <v>-45.769999999999982</v>
+        <v>1942.23</v>
       </c>
       <c r="AT64" s="45">
         <f t="shared" si="36"/>
-        <v>-167.56</v>
+        <v>17.75</v>
       </c>
       <c r="AU64" s="45">
         <f t="shared" si="37"/>
-        <v>-61.42</v>
+        <v>6.8299999999999983</v>
       </c>
       <c r="AV64" s="45">
         <f t="shared" si="65"/>
-        <v>501</v>
+        <v>20</v>
       </c>
       <c r="AW64" s="25">
         <v>15</v>
@@ -15561,39 +15758,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC64" s="11"/>
-      <c r="BD64" s="46"/>
-      <c r="BE64" s="22"/>
+      <c r="BD64" s="46">
+        <f>BM64*24*60/BH64</f>
+        <v>8.8967442096820649E-3</v>
+      </c>
+      <c r="BE64" s="22">
+        <f>BP64/BH64</f>
+        <v>5.5208033108114681E-3</v>
+      </c>
       <c r="BF64" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.068519603E-2</v>
       </c>
       <c r="BG64" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15.386682283200003</v>
       </c>
       <c r="BH64" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI64" s="47" t="str">
+        <v>1845.4569999999999</v>
+      </c>
+      <c r="BI64" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ64" s="47" t="str">
+        <v>0.10041415215851685</v>
+      </c>
+      <c r="BJ64" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.10900588235294117</v>
       </c>
       <c r="BK64" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>16.418558878967232</v>
       </c>
       <c r="BL64" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM64" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.1401776999282799E-2</v>
       </c>
       <c r="BN64" s="48" t="str">
         <f t="shared" si="32"/>
@@ -15604,20 +15806,19 @@
         <v/>
       </c>
       <c r="BP64" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>10.188405115560199</v>
       </c>
       <c r="BQ64" s="28">
         <f t="shared" ref="BQ64:BQ68" si="80">IF(BL64&lt;&gt;"",BL64/0.000385,IF(BM64&lt;&gt;"",BM64/0.000385,BN64/0.000385))</f>
-        <v>0</v>
+        <v>29.615005192942338</v>
       </c>
       <c r="BR64" s="49">
         <f t="shared" ref="BR64:BR68" si="81">IF(BL64&lt;&gt;"",BL64,IF(BM64&lt;&gt;"",BM64,BN64))</f>
-        <v>0</v>
+        <v>1.1401776999282799E-2</v>
       </c>
       <c r="BS64" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>10.188405115560199</v>
       </c>
     </row>
     <row r="65" spans="1:71" x14ac:dyDescent="0.3">
@@ -15633,70 +15834,135 @@
       <c r="D65">
         <v>10</v>
       </c>
-      <c r="F65" s="61"/>
+      <c r="F65" s="61">
+        <v>45543.423032407401</v>
+      </c>
       <c r="G65" s="64">
         <v>5497.99</v>
       </c>
       <c r="H65" s="44"/>
       <c r="I65" s="44"/>
-      <c r="J65" s="44"/>
-      <c r="K65" s="44"/>
-      <c r="L65" s="44"/>
-      <c r="M65" s="44"/>
-      <c r="N65" s="44"/>
-      <c r="O65" s="44"/>
-      <c r="P65" s="44"/>
-      <c r="Q65" s="44"/>
+      <c r="J65" s="44">
+        <v>20.2</v>
+      </c>
+      <c r="K65" s="44">
+        <v>18</v>
+      </c>
+      <c r="L65" s="44">
+        <v>89.1</v>
+      </c>
+      <c r="M65" s="44">
+        <v>19.2</v>
+      </c>
+      <c r="N65" s="44">
+        <v>438</v>
+      </c>
+      <c r="O65" s="44">
+        <v>2.36</v>
+      </c>
+      <c r="P65" s="44">
+        <v>0.22</v>
+      </c>
+      <c r="Q65" s="44">
+        <v>3.22</v>
+      </c>
       <c r="R65" s="44"/>
-      <c r="S65" s="44"/>
-      <c r="T65" s="44"/>
-      <c r="U65" s="44"/>
-      <c r="V65" s="44"/>
-      <c r="W65" s="44"/>
-      <c r="X65" s="44"/>
-      <c r="Y65" s="44"/>
-      <c r="Z65" s="44"/>
-      <c r="AA65" s="44"/>
-      <c r="AB65" s="44"/>
-      <c r="AC65" s="44"/>
-      <c r="AD65" s="17"/>
-      <c r="AE65" s="44"/>
-      <c r="AF65" s="44"/>
-      <c r="AG65" s="44"/>
+      <c r="S65" s="44">
+        <v>0.78</v>
+      </c>
+      <c r="T65" s="44">
+        <v>2.21</v>
+      </c>
+      <c r="U65" s="44">
+        <v>2.19</v>
+      </c>
+      <c r="V65" s="44">
+        <v>7.2469999999999999</v>
+      </c>
+      <c r="W65" s="44">
+        <v>118.5</v>
+      </c>
+      <c r="X65" s="44">
+        <v>46.8</v>
+      </c>
+      <c r="Y65" s="44">
+        <v>1.5</v>
+      </c>
+      <c r="Z65" s="44">
+        <v>176.3</v>
+      </c>
+      <c r="AA65" s="44">
+        <v>50.2</v>
+      </c>
+      <c r="AB65" s="44">
+        <v>104</v>
+      </c>
+      <c r="AC65" s="44">
+        <v>37.9</v>
+      </c>
+      <c r="AD65" s="17">
+        <v>7.2880000000000003</v>
+      </c>
+      <c r="AE65" s="44">
+        <v>298</v>
+      </c>
+      <c r="AF65" s="44">
+        <v>50.4</v>
+      </c>
+      <c r="AG65" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH65" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI65" s="44"/>
-      <c r="AJ65" s="44"/>
-      <c r="AK65" s="44"/>
-      <c r="AL65" s="44"/>
+        <v>0.504</v>
+      </c>
+      <c r="AI65" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ65" s="44">
+        <v>38.045999999999999</v>
+      </c>
+      <c r="AK65" s="44">
+        <v>5.1144999999999996</v>
+      </c>
+      <c r="AL65" s="44">
+        <f>AL53+1.87</f>
+        <v>8.5300000000000011</v>
+      </c>
       <c r="AM65" s="45">
         <f t="shared" si="79"/>
-        <v>0</v>
-      </c>
-      <c r="AN65" s="44"/>
-      <c r="AO65" s="44"/>
-      <c r="AP65" s="44"/>
-      <c r="AQ65" s="44"/>
+        <v>2.08588154275034E-2</v>
+      </c>
+      <c r="AN65" s="44">
+        <v>249.44</v>
+      </c>
+      <c r="AO65" s="44">
+        <v>84.76</v>
+      </c>
+      <c r="AP65" s="44">
+        <v>384</v>
+      </c>
+      <c r="AQ65" s="44">
+        <v>2061</v>
+      </c>
       <c r="AR65" s="45">
         <v>84.700000000000045</v>
       </c>
       <c r="AS65" s="45">
         <f t="shared" si="60"/>
-        <v>-84.700000000000045</v>
+        <v>1976.3</v>
       </c>
       <c r="AT65" s="45">
         <f t="shared" si="36"/>
-        <v>-211.31</v>
+        <v>38.129999999999995</v>
       </c>
       <c r="AU65" s="45">
         <f t="shared" si="37"/>
-        <v>-76.27</v>
+        <v>8.4900000000000091</v>
       </c>
       <c r="AV65" s="45">
         <f t="shared" si="65"/>
-        <v>430</v>
+        <v>46</v>
       </c>
       <c r="AW65" s="25">
         <v>15</v>
@@ -15717,39 +15983,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC65" s="11"/>
-      <c r="BD65" s="46"/>
-      <c r="BE65" s="22"/>
+      <c r="BD65" s="46">
+        <f>BM65*24*60/BH65</f>
+        <v>1.5636859162771067E-2</v>
+      </c>
+      <c r="BE65" s="22">
+        <f>BP65/BH65</f>
+        <v>1.6524849493275854E-3</v>
+      </c>
       <c r="BF65" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.0372808699999998E-2</v>
       </c>
       <c r="BG65" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.936844527999996</v>
       </c>
       <c r="BH65" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI65" s="47" t="str">
+        <v>1920.8905</v>
+      </c>
+      <c r="BI65" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ65" s="47" t="str">
+        <v>0.12985643897973362</v>
+      </c>
+      <c r="BJ65" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.14672941176470589</v>
       </c>
       <c r="BK65" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>30.036694215604896</v>
       </c>
       <c r="BL65" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM65" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>2.08588154275034E-2</v>
       </c>
       <c r="BN65" s="48" t="str">
         <f t="shared" si="32"/>
@@ -15760,20 +16031,19 @@
         <v/>
       </c>
       <c r="BP65" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>3.17424264055634</v>
       </c>
       <c r="BQ65" s="28">
         <f t="shared" si="80"/>
-        <v>0</v>
+        <v>54.178741370138702</v>
       </c>
       <c r="BR65" s="49">
         <f t="shared" si="81"/>
-        <v>0</v>
+        <v>2.08588154275034E-2</v>
       </c>
       <c r="BS65" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>3.17424264055634</v>
       </c>
     </row>
     <row r="66" spans="1:71" x14ac:dyDescent="0.3">
@@ -15789,70 +16059,135 @@
       <c r="D66">
         <v>10</v>
       </c>
-      <c r="F66" s="61"/>
+      <c r="F66" s="61">
+        <v>45543.425671296303</v>
+      </c>
       <c r="G66" s="64">
         <v>5497.99</v>
       </c>
       <c r="H66" s="44"/>
       <c r="I66" s="44"/>
-      <c r="J66" s="44"/>
-      <c r="K66" s="44"/>
-      <c r="L66" s="44"/>
-      <c r="M66" s="44"/>
-      <c r="N66" s="44"/>
-      <c r="O66" s="44"/>
-      <c r="P66" s="44"/>
-      <c r="Q66" s="44"/>
+      <c r="J66" s="44">
+        <v>20.2</v>
+      </c>
+      <c r="K66" s="44">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="L66" s="44">
+        <v>89.7</v>
+      </c>
+      <c r="M66" s="44">
+        <v>19</v>
+      </c>
+      <c r="N66" s="44">
+        <v>430</v>
+      </c>
+      <c r="O66" s="44">
+        <v>1.71</v>
+      </c>
+      <c r="P66" s="44">
+        <v>0.21</v>
+      </c>
+      <c r="Q66" s="44">
+        <v>1.31</v>
+      </c>
       <c r="R66" s="44"/>
-      <c r="S66" s="44"/>
-      <c r="T66" s="44"/>
-      <c r="U66" s="44"/>
-      <c r="V66" s="44"/>
-      <c r="W66" s="44"/>
-      <c r="X66" s="44"/>
-      <c r="Y66" s="44"/>
-      <c r="Z66" s="44"/>
-      <c r="AA66" s="44"/>
-      <c r="AB66" s="44"/>
-      <c r="AC66" s="44"/>
-      <c r="AD66" s="17"/>
-      <c r="AE66" s="44"/>
-      <c r="AF66" s="44"/>
-      <c r="AG66" s="44"/>
+      <c r="S66" s="44">
+        <v>0.6</v>
+      </c>
+      <c r="T66" s="44">
+        <v>2.08</v>
+      </c>
+      <c r="U66" s="44">
+        <v>2.54</v>
+      </c>
+      <c r="V66" s="44">
+        <v>7.2779999999999996</v>
+      </c>
+      <c r="W66" s="44">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="X66" s="44">
+        <v>30</v>
+      </c>
+      <c r="Y66" s="44">
+        <v>1.48</v>
+      </c>
+      <c r="Z66" s="44">
+        <v>183.1</v>
+      </c>
+      <c r="AA66" s="44">
+        <v>58.4</v>
+      </c>
+      <c r="AB66" s="44">
+        <v>112.5</v>
+      </c>
+      <c r="AC66" s="44">
+        <v>24.3</v>
+      </c>
+      <c r="AD66" s="17">
+        <v>7.319</v>
+      </c>
+      <c r="AE66" s="44">
+        <v>301</v>
+      </c>
+      <c r="AF66" s="44">
+        <v>51.1</v>
+      </c>
+      <c r="AG66" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH66" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI66" s="44"/>
-      <c r="AJ66" s="44"/>
-      <c r="AK66" s="44"/>
-      <c r="AL66" s="44"/>
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="AI66" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ66" s="44">
+        <v>43.091000000000001</v>
+      </c>
+      <c r="AK66" s="44">
+        <v>13.548</v>
+      </c>
+      <c r="AL66" s="44">
+        <f>AL54+1.91</f>
+        <v>8.67</v>
+      </c>
       <c r="AM66" s="45">
         <f t="shared" si="79"/>
         <v>0</v>
       </c>
-      <c r="AN66" s="44"/>
-      <c r="AO66" s="44"/>
-      <c r="AP66" s="44"/>
-      <c r="AQ66" s="44"/>
+      <c r="AN66" s="44">
+        <v>233.93</v>
+      </c>
+      <c r="AO66" s="44">
+        <v>70.87</v>
+      </c>
+      <c r="AP66" s="44">
+        <v>406</v>
+      </c>
+      <c r="AQ66" s="44">
+        <v>2044</v>
+      </c>
       <c r="AR66" s="45">
         <v>47.420000000000073</v>
       </c>
       <c r="AS66" s="45">
-        <f t="shared" si="60"/>
-        <v>-47.420000000000073</v>
+        <f>AQ66-AR66</f>
+        <v>1996.58</v>
       </c>
       <c r="AT66" s="45">
         <f t="shared" si="36"/>
-        <v>-204.07</v>
+        <v>29.860000000000014</v>
       </c>
       <c r="AU66" s="45">
         <f t="shared" si="37"/>
-        <v>-70.87</v>
+        <v>0</v>
       </c>
       <c r="AV66" s="45">
         <f t="shared" si="65"/>
-        <v>443</v>
+        <v>37</v>
       </c>
       <c r="AW66" s="25">
         <v>15</v>
@@ -15876,23 +16211,23 @@
       <c r="BE66" s="22"/>
       <c r="BF66" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.034474187E-2</v>
       </c>
       <c r="BG66" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.8964282928</v>
       </c>
       <c r="BH66" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI66" s="47" t="str">
+        <v>1905.1089999999999</v>
+      </c>
+      <c r="BI66" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ66" s="47" t="str">
+        <v>0.12279087443290647</v>
+      </c>
+      <c r="BJ66" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.13760588235294119</v>
       </c>
       <c r="BK66" s="47">
         <f t="shared" si="18"/>
@@ -15912,7 +16247,7 @@
       </c>
       <c r="BO66" s="47">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>8.0490855249999989</v>
       </c>
       <c r="BP66" s="51" t="str">
         <f t="shared" si="28"/>
@@ -15928,7 +16263,7 @@
       </c>
       <c r="BS66" s="30">
         <f t="shared" si="21"/>
-        <v>11.512499999999999</v>
+        <v>8.0490855249999989</v>
       </c>
     </row>
     <row r="67" spans="1:71" x14ac:dyDescent="0.3">
@@ -15944,70 +16279,131 @@
       <c r="D67">
         <v>10</v>
       </c>
-      <c r="F67" s="61"/>
+      <c r="F67" s="61">
+        <v>45543.428912037001</v>
+      </c>
       <c r="G67" s="64">
         <v>5497.99</v>
       </c>
       <c r="H67" s="44"/>
       <c r="I67" s="44"/>
-      <c r="J67" s="44"/>
-      <c r="K67" s="44"/>
-      <c r="L67" s="44"/>
-      <c r="M67" s="44"/>
-      <c r="N67" s="44"/>
+      <c r="J67" s="44">
+        <v>21.1</v>
+      </c>
+      <c r="K67" s="44">
+        <v>8.32</v>
+      </c>
+      <c r="L67" s="44">
+        <v>39.5</v>
+      </c>
+      <c r="M67" s="44">
+        <v>15.6</v>
+      </c>
+      <c r="N67" s="44">
+        <v>818</v>
+      </c>
       <c r="O67" s="44"/>
-      <c r="P67" s="44"/>
-      <c r="Q67" s="44"/>
+      <c r="P67" s="44">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="Q67" s="44">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="R67" s="44"/>
-      <c r="S67" s="44"/>
-      <c r="T67" s="44"/>
+      <c r="S67" s="44">
+        <v>0.75</v>
+      </c>
+      <c r="T67" s="44">
+        <v>3.48</v>
+      </c>
       <c r="U67" s="44"/>
-      <c r="V67" s="44"/>
-      <c r="W67" s="44"/>
-      <c r="X67" s="44"/>
-      <c r="Y67" s="44"/>
-      <c r="Z67" s="44"/>
-      <c r="AA67" s="44"/>
-      <c r="AB67" s="44"/>
-      <c r="AC67" s="44"/>
-      <c r="AD67" s="17"/>
-      <c r="AE67" s="44"/>
-      <c r="AF67" s="44"/>
-      <c r="AG67" s="44"/>
+      <c r="V67" s="44">
+        <v>7.032</v>
+      </c>
+      <c r="W67" s="44">
+        <v>66.3</v>
+      </c>
+      <c r="X67" s="44">
+        <v>86</v>
+      </c>
+      <c r="Y67" s="44">
+        <v>7.2</v>
+      </c>
+      <c r="Z67" s="44">
+        <v>327.9</v>
+      </c>
+      <c r="AA67" s="44">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="AB67" s="44">
+        <v>58.1</v>
+      </c>
+      <c r="AC67" s="44">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="AD67" s="17">
+        <v>7.069</v>
+      </c>
+      <c r="AE67" s="44">
+        <v>301</v>
+      </c>
+      <c r="AF67" s="44">
+        <v>45.2</v>
+      </c>
+      <c r="AG67" s="44">
+        <v>7.09</v>
+      </c>
       <c r="AH67" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI67" s="44"/>
-      <c r="AJ67" s="44"/>
-      <c r="AK67" s="44"/>
-      <c r="AL67" s="44"/>
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="AI67" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ67" s="44">
+        <v>157.88999999999999</v>
+      </c>
+      <c r="AK67" s="44">
+        <v>7.3125999999999998</v>
+      </c>
+      <c r="AL67" s="44">
+        <f>AL55+1.84</f>
+        <v>8.2800000000000011</v>
+      </c>
       <c r="AM67" s="45">
         <f t="shared" si="79"/>
         <v>0</v>
       </c>
-      <c r="AN67" s="44"/>
-      <c r="AO67" s="44"/>
-      <c r="AP67" s="44"/>
-      <c r="AQ67" s="44"/>
+      <c r="AN67" s="44">
+        <v>261.68</v>
+      </c>
+      <c r="AO67" s="44">
+        <v>77.819999999999993</v>
+      </c>
+      <c r="AP67" s="44">
+        <v>353</v>
+      </c>
+      <c r="AQ67" s="44">
+        <v>2185</v>
+      </c>
       <c r="AR67" s="45">
         <v>133.55999999999995</v>
       </c>
       <c r="AS67" s="45">
-        <f t="shared" ref="AS67:AS80" si="82">AQ67-AR67</f>
-        <v>-133.55999999999995</v>
+        <f>AQ67-AR67</f>
+        <v>2051.44</v>
       </c>
       <c r="AT67" s="45">
         <f t="shared" si="36"/>
-        <v>-227.05</v>
+        <v>34.629999999999995</v>
       </c>
       <c r="AU67" s="45">
         <f t="shared" si="37"/>
-        <v>-77.819999999999993</v>
+        <v>0</v>
       </c>
       <c r="AV67" s="45">
         <f t="shared" si="65"/>
-        <v>394</v>
+        <v>41</v>
       </c>
       <c r="AW67" s="25">
         <v>15</v>
@@ -16030,27 +16426,27 @@
       <c r="BC67" s="11"/>
       <c r="BE67" s="22"/>
       <c r="BF67" s="11">
-        <f t="shared" ref="BF67:BF74" si="83">BB67*K67*BH67/1000</f>
-        <v>0</v>
+        <f t="shared" ref="BF67:BF74" si="82">BB67*K67*BH67/1000</f>
+        <v>5.1117645696000013E-3</v>
       </c>
       <c r="BG67" s="46">
-        <f t="shared" ref="BG67:BG74" si="84">BF67*24*60</f>
-        <v>0</v>
+        <f t="shared" ref="BG67:BG74" si="83">BF67*24*60</f>
+        <v>7.3609409802240027</v>
       </c>
       <c r="BH67" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI67" s="47" t="str">
+        <v>2047.9826000000003</v>
+      </c>
+      <c r="BI67" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ67" s="47" t="str">
+        <v>0.12777452308432696</v>
+      </c>
+      <c r="BJ67" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.1539294117647059</v>
       </c>
       <c r="BK67" s="47">
-        <f t="shared" ref="BK67:BK74" si="85">AM67*24*60</f>
+        <f t="shared" ref="BK67:BK74" si="84">AM67*24*60</f>
         <v>0</v>
       </c>
       <c r="BL67" s="47">
@@ -16062,12 +16458,12 @@
         <v/>
       </c>
       <c r="BN67" s="48" t="str">
-        <f t="shared" ref="BN67:BN74" si="86">IF(B67="No MPC", BB67*K67*BH67/1000,"")</f>
+        <f t="shared" ref="BN67:BN74" si="85">IF(B67="No MPC", BB67*K67*BH67/1000,"")</f>
         <v/>
       </c>
       <c r="BO67" s="47">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>15.001472545000004</v>
       </c>
       <c r="BP67" s="51" t="str">
         <f t="shared" si="28"/>
@@ -16082,8 +16478,8 @@
         <v>0</v>
       </c>
       <c r="BS67" s="30">
-        <f t="shared" ref="BS67:BS74" si="87">IF(BO67&lt;&gt;"",BO67,BP67)</f>
-        <v>11.512499999999999</v>
+        <f t="shared" ref="BS67:BS74" si="86">IF(BO67&lt;&gt;"",BO67,BP67)</f>
+        <v>15.001472545000004</v>
       </c>
     </row>
     <row r="68" spans="1:71" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -16100,70 +16496,135 @@
         <v>10</v>
       </c>
       <c r="E68" s="5"/>
-      <c r="F68" s="62"/>
+      <c r="F68" s="62">
+        <v>45543.4315740741</v>
+      </c>
       <c r="G68" s="65">
         <v>5497.99</v>
       </c>
       <c r="H68" s="7"/>
       <c r="I68" s="7"/>
-      <c r="J68" s="7"/>
-      <c r="K68" s="7"/>
-      <c r="L68" s="7"/>
-      <c r="M68" s="7"/>
-      <c r="N68" s="7"/>
-      <c r="O68" s="7"/>
-      <c r="P68" s="7"/>
-      <c r="Q68" s="7"/>
+      <c r="J68" s="7">
+        <v>21.5</v>
+      </c>
+      <c r="K68" s="7">
+        <v>19.7</v>
+      </c>
+      <c r="L68" s="7">
+        <v>92</v>
+      </c>
+      <c r="M68" s="7">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="N68" s="7">
+        <v>367</v>
+      </c>
+      <c r="O68" s="7">
+        <v>1.57</v>
+      </c>
+      <c r="P68" s="7">
+        <v>0.19</v>
+      </c>
+      <c r="Q68" s="7">
+        <v>0.66</v>
+      </c>
       <c r="R68" s="7"/>
-      <c r="S68" s="7"/>
-      <c r="T68" s="7"/>
-      <c r="U68" s="7"/>
-      <c r="V68" s="7"/>
-      <c r="W68" s="7"/>
-      <c r="X68" s="7"/>
-      <c r="Y68" s="7"/>
-      <c r="Z68" s="7"/>
-      <c r="AA68" s="7"/>
-      <c r="AB68" s="7"/>
-      <c r="AC68" s="7"/>
-      <c r="AD68" s="18"/>
-      <c r="AE68" s="7"/>
-      <c r="AF68" s="7"/>
-      <c r="AG68" s="7"/>
+      <c r="S68" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="T68" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="U68" s="7">
+        <v>0.73</v>
+      </c>
+      <c r="V68" s="7">
+        <v>7.2640000000000002</v>
+      </c>
+      <c r="W68" s="7">
+        <v>120.2</v>
+      </c>
+      <c r="X68" s="7">
+        <v>31.7</v>
+      </c>
+      <c r="Y68" s="7">
+        <v>1.79</v>
+      </c>
+      <c r="Z68" s="7">
+        <v>160</v>
+      </c>
+      <c r="AA68" s="7">
+        <v>53</v>
+      </c>
+      <c r="AB68" s="7">
+        <v>105.4</v>
+      </c>
+      <c r="AC68" s="7">
+        <v>25.6</v>
+      </c>
+      <c r="AD68" s="18">
+        <v>7.3049999999999997</v>
+      </c>
+      <c r="AE68" s="7">
+        <v>299</v>
+      </c>
+      <c r="AF68" s="7">
+        <v>49.3</v>
+      </c>
+      <c r="AG68" s="7">
+        <v>7.3</v>
+      </c>
       <c r="AH68" s="41">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI68" s="7"/>
-      <c r="AJ68" s="7"/>
-      <c r="AK68" s="7"/>
-      <c r="AL68" s="7"/>
+        <v>0.49299999999999999</v>
+      </c>
+      <c r="AI68" s="7">
+        <v>34</v>
+      </c>
+      <c r="AJ68" s="7">
+        <v>28.271000000000001</v>
+      </c>
+      <c r="AK68" s="7">
+        <v>45.024999999999999</v>
+      </c>
+      <c r="AL68" s="7">
+        <f>AL56+1.86</f>
+        <v>8.379999999999999</v>
+      </c>
       <c r="AM68" s="41">
         <f t="shared" si="79"/>
         <v>0</v>
       </c>
-      <c r="AN68" s="7"/>
-      <c r="AO68" s="7"/>
-      <c r="AP68" s="7"/>
-      <c r="AQ68" s="7"/>
+      <c r="AN68" s="7">
+        <v>201.93</v>
+      </c>
+      <c r="AO68" s="7">
+        <v>69.75</v>
+      </c>
+      <c r="AP68" s="7">
+        <v>460</v>
+      </c>
+      <c r="AQ68" s="7">
+        <v>2025</v>
+      </c>
       <c r="AR68" s="41">
         <v>51.660000000000082</v>
       </c>
       <c r="AS68" s="41">
-        <f t="shared" si="82"/>
-        <v>-51.660000000000082</v>
+        <f>AQ68-AR68</f>
+        <v>1973.34</v>
       </c>
       <c r="AT68" s="41">
         <f t="shared" si="36"/>
-        <v>-187.96</v>
+        <v>13.969999999999999</v>
       </c>
       <c r="AU68" s="41">
         <f t="shared" si="37"/>
-        <v>-56.59</v>
+        <v>13.159999999999997</v>
       </c>
       <c r="AV68" s="41">
         <f t="shared" si="65"/>
-        <v>476</v>
+        <v>16</v>
       </c>
       <c r="AW68" s="26">
         <v>15</v>
@@ -16187,31 +16648,31 @@
       <c r="BD68" s="5"/>
       <c r="BE68" s="23"/>
       <c r="BF68" s="12">
+        <f t="shared" si="82"/>
+        <v>1.1160183959999999E-2</v>
+      </c>
+      <c r="BG68" s="13">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG68" s="13">
-        <f t="shared" si="84"/>
-        <v>0</v>
+        <v>16.070664902399997</v>
       </c>
       <c r="BH68" s="13">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI68" s="14" t="str">
-        <f t="shared" ref="BI68:BI80" si="88">IF(ISBLANK(AN68),"",IFERROR(AN68/BH68,0))</f>
-        <v/>
-      </c>
-      <c r="BJ68" s="14" t="str">
-        <f t="shared" ref="BJ68:BJ80" si="89">IF(ISBLANK(AN68),"",AN68/AX68)</f>
-        <v/>
+        <v>1888.3559999999998</v>
+      </c>
+      <c r="BI68" s="14">
+        <f t="shared" ref="BI68:BI80" si="87">IF(ISBLANK(AN68),"",IFERROR(AN68/BH68,0))</f>
+        <v>0.10693428569612935</v>
+      </c>
+      <c r="BJ68" s="14">
+        <f t="shared" ref="BJ68:BJ80" si="88">IF(ISBLANK(AN68),"",AN68/AX68)</f>
+        <v>0.11878235294117648</v>
       </c>
       <c r="BK68" s="14">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BL68" s="14">
-        <f t="shared" ref="BL68:BL80" si="90">IF(B68="Python",BC68*BH68/24/60,"")</f>
+        <f t="shared" ref="BL68:BL80" si="89">IF(B68="Python",BC68*BH68/24/60,"")</f>
         <v>0</v>
       </c>
       <c r="BM68" s="48" t="str">
@@ -16219,12 +16680,12 @@
         <v/>
       </c>
       <c r="BN68" s="36" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO68" s="14">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>11.046882599999998</v>
       </c>
       <c r="BP68" s="52" t="str">
         <f t="shared" si="28"/>
@@ -16239,8 +16700,8 @@
         <v>0</v>
       </c>
       <c r="BS68" s="31">
-        <f t="shared" si="87"/>
-        <v>11.512499999999999</v>
+        <f t="shared" si="86"/>
+        <v>11.046882599999998</v>
       </c>
     </row>
     <row r="69" spans="1:71" x14ac:dyDescent="0.3">
@@ -16307,20 +16768,20 @@
         <v>137.11999999999989</v>
       </c>
       <c r="AS69" s="40">
-        <f t="shared" si="82"/>
+        <f t="shared" ref="AS67:AS80" si="90">AQ69-AR69</f>
         <v>-137.11999999999989</v>
       </c>
       <c r="AT69" s="40">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>-169.89</v>
       </c>
       <c r="AU69" s="40">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>-65.31</v>
       </c>
       <c r="AV69" s="40">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>497</v>
       </c>
       <c r="AW69" s="24">
         <v>15</v>
@@ -16344,11 +16805,11 @@
       <c r="BD69" s="9"/>
       <c r="BE69" s="21"/>
       <c r="BF69" s="8">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG69" s="9">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG69" s="9">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH69" s="9">
@@ -16356,19 +16817,19 @@
         <v>1520</v>
       </c>
       <c r="BI69" s="10" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ69" s="10" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ69" s="10" t="str">
+      <c r="BK69" s="10">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL69" s="10" t="str">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK69" s="10">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL69" s="10" t="str">
-        <f t="shared" si="90"/>
         <v/>
       </c>
       <c r="BM69" s="10">
@@ -16376,7 +16837,7 @@
         <v>0</v>
       </c>
       <c r="BN69" s="35" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO69" s="10" t="str">
@@ -16396,7 +16857,7 @@
         <v>0</v>
       </c>
       <c r="BS69" s="32">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
     </row>
@@ -16463,20 +16924,20 @@
         <v>45.769999999999982</v>
       </c>
       <c r="AS70" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-45.769999999999982</v>
       </c>
       <c r="AT70" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>-185.31</v>
       </c>
       <c r="AU70" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>-68.25</v>
       </c>
       <c r="AV70" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>481</v>
       </c>
       <c r="AW70" s="25">
         <v>15</v>
@@ -16500,11 +16961,11 @@
       <c r="BD70" s="46"/>
       <c r="BE70" s="22"/>
       <c r="BF70" s="11">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG70" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG70" s="46">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH70" s="46">
@@ -16512,19 +16973,19 @@
         <v>1520</v>
       </c>
       <c r="BI70" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ70" s="47" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ70" s="47" t="str">
+      <c r="BK70" s="47">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL70" s="47" t="str">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK70" s="47">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL70" s="47" t="str">
-        <f t="shared" si="90"/>
         <v/>
       </c>
       <c r="BM70" s="47">
@@ -16532,7 +16993,7 @@
         <v>0</v>
       </c>
       <c r="BN70" s="48" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO70" s="47" t="str">
@@ -16552,7 +17013,7 @@
         <v>0</v>
       </c>
       <c r="BS70" s="30">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
     </row>
@@ -16619,20 +17080,20 @@
         <v>84.700000000000045</v>
       </c>
       <c r="AS71" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-84.700000000000045</v>
       </c>
       <c r="AT71" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>-249.44</v>
       </c>
       <c r="AU71" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>-84.76</v>
       </c>
       <c r="AV71" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="AW71" s="25">
         <v>15</v>
@@ -16656,11 +17117,11 @@
       <c r="BD71" s="46"/>
       <c r="BE71" s="22"/>
       <c r="BF71" s="11">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG71" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG71" s="46">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH71" s="46">
@@ -16668,19 +17129,19 @@
         <v>1520</v>
       </c>
       <c r="BI71" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ71" s="47" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ71" s="47" t="str">
+      <c r="BK71" s="47">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL71" s="47" t="str">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK71" s="47">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL71" s="47" t="str">
-        <f t="shared" si="90"/>
         <v/>
       </c>
       <c r="BM71" s="47">
@@ -16688,7 +17149,7 @@
         <v>0</v>
       </c>
       <c r="BN71" s="48" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO71" s="47" t="str">
@@ -16708,7 +17169,7 @@
         <v>0</v>
       </c>
       <c r="BS71" s="30">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0</v>
       </c>
     </row>
@@ -16775,20 +17236,20 @@
         <v>47.420000000000073</v>
       </c>
       <c r="AS72" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-47.420000000000073</v>
       </c>
       <c r="AT72" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>-233.93</v>
       </c>
       <c r="AU72" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>-70.87</v>
       </c>
       <c r="AV72" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>406</v>
       </c>
       <c r="AW72" s="25">
         <v>15</v>
@@ -16811,11 +17272,11 @@
       <c r="BC72" s="11"/>
       <c r="BE72" s="22"/>
       <c r="BF72" s="11">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG72" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG72" s="46">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH72" s="46">
@@ -16823,19 +17284,19 @@
         <v>1520</v>
       </c>
       <c r="BI72" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ72" s="47" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ72" s="47" t="str">
+      <c r="BK72" s="47">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL72" s="47">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK72" s="47">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL72" s="47">
-        <f t="shared" si="90"/>
         <v>0</v>
       </c>
       <c r="BM72" s="48" t="str">
@@ -16843,7 +17304,7 @@
         <v/>
       </c>
       <c r="BN72" s="48" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO72" s="47">
@@ -16863,7 +17324,7 @@
         <v>0</v>
       </c>
       <c r="BS72" s="30">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>11.4</v>
       </c>
     </row>
@@ -16930,20 +17391,20 @@
         <v>133.55999999999995</v>
       </c>
       <c r="AS73" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-133.55999999999995</v>
       </c>
       <c r="AT73" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>-261.68</v>
       </c>
       <c r="AU73" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>-77.819999999999993</v>
       </c>
       <c r="AV73" s="45">
         <f t="shared" ref="AV73:AV80" si="98">AP67-AP73</f>
-        <v>0</v>
+        <v>353</v>
       </c>
       <c r="AW73" s="25">
         <v>15</v>
@@ -16966,11 +17427,11 @@
       <c r="BC73" s="11"/>
       <c r="BE73" s="22"/>
       <c r="BF73" s="11">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG73" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG73" s="46">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH73" s="46">
@@ -16978,19 +17439,19 @@
         <v>1520</v>
       </c>
       <c r="BI73" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ73" s="47" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ73" s="47" t="str">
+      <c r="BK73" s="47">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL73" s="47">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK73" s="47">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL73" s="47">
-        <f t="shared" si="90"/>
         <v>0</v>
       </c>
       <c r="BM73" s="48" t="str">
@@ -16998,7 +17459,7 @@
         <v/>
       </c>
       <c r="BN73" s="48" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO73" s="47">
@@ -17018,7 +17479,7 @@
         <v>0</v>
       </c>
       <c r="BS73" s="30">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>11.4</v>
       </c>
     </row>
@@ -17086,20 +17547,20 @@
         <v>51.660000000000082</v>
       </c>
       <c r="AS74" s="41">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-51.660000000000082</v>
       </c>
       <c r="AT74" s="41">
         <f t="shared" ref="AT74:AT80" si="99">AN74-AN68</f>
-        <v>0</v>
+        <v>-201.93</v>
       </c>
       <c r="AU74" s="41">
         <f t="shared" ref="AU74:AU80" si="100">AO74-AO68</f>
-        <v>0</v>
+        <v>-69.75</v>
       </c>
       <c r="AV74" s="41">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>460</v>
       </c>
       <c r="AW74" s="26">
         <v>15</v>
@@ -17123,11 +17584,11 @@
       <c r="BD74" s="5"/>
       <c r="BE74" s="23"/>
       <c r="BF74" s="12">
+        <f t="shared" si="82"/>
+        <v>0</v>
+      </c>
+      <c r="BG74" s="13">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG74" s="13">
-        <f t="shared" si="84"/>
         <v>0</v>
       </c>
       <c r="BH74" s="13">
@@ -17135,19 +17596,19 @@
         <v>1520</v>
       </c>
       <c r="BI74" s="14" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ74" s="14" t="str">
         <f t="shared" si="88"/>
         <v/>
       </c>
-      <c r="BJ74" s="14" t="str">
+      <c r="BK74" s="14">
+        <f t="shared" si="84"/>
+        <v>0</v>
+      </c>
+      <c r="BL74" s="14">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK74" s="14">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL74" s="14">
-        <f t="shared" si="90"/>
         <v>0</v>
       </c>
       <c r="BM74" s="48" t="str">
@@ -17155,7 +17616,7 @@
         <v/>
       </c>
       <c r="BN74" s="36" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO74" s="14">
@@ -17175,7 +17636,7 @@
         <v>0</v>
       </c>
       <c r="BS74" s="31">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>11.4</v>
       </c>
     </row>
@@ -17243,7 +17704,7 @@
         <v>137.11999999999989</v>
       </c>
       <c r="AS75" s="40">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-137.11999999999989</v>
       </c>
       <c r="AT75" s="40">
@@ -17292,11 +17753,11 @@
         <v>1505</v>
       </c>
       <c r="BI75" s="10" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ75" s="10" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ75" s="10" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK75" s="10">
@@ -17304,7 +17765,7 @@
         <v>0</v>
       </c>
       <c r="BL75" s="10" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM75" s="10">
@@ -17399,7 +17860,7 @@
         <v>45.769999999999982</v>
       </c>
       <c r="AS76" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-45.769999999999982</v>
       </c>
       <c r="AT76" s="45">
@@ -17448,11 +17909,11 @@
         <v>1505</v>
       </c>
       <c r="BI76" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ76" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ76" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK76" s="47">
@@ -17460,7 +17921,7 @@
         <v>0</v>
       </c>
       <c r="BL76" s="47" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM76" s="47">
@@ -17555,7 +18016,7 @@
         <v>84.700000000000045</v>
       </c>
       <c r="AS77" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-84.700000000000045</v>
       </c>
       <c r="AT77" s="45">
@@ -17604,11 +18065,11 @@
         <v>1505</v>
       </c>
       <c r="BI77" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ77" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ77" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK77" s="47">
@@ -17616,7 +18077,7 @@
         <v>0</v>
       </c>
       <c r="BL77" s="47" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM77" s="47">
@@ -17711,7 +18172,7 @@
         <v>47.420000000000073</v>
       </c>
       <c r="AS78" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-47.420000000000073</v>
       </c>
       <c r="AT78" s="45">
@@ -17759,11 +18220,11 @@
         <v>1505</v>
       </c>
       <c r="BI78" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ78" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ78" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK78" s="47">
@@ -17771,7 +18232,7 @@
         <v>0</v>
       </c>
       <c r="BL78" s="47">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM78" s="48" t="str">
@@ -17866,7 +18327,7 @@
         <v>133.55999999999995</v>
       </c>
       <c r="AS79" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-133.55999999999995</v>
       </c>
       <c r="AT79" s="45">
@@ -17914,11 +18375,11 @@
         <v>1505</v>
       </c>
       <c r="BI79" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ79" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ79" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK79" s="47">
@@ -17926,7 +18387,7 @@
         <v>0</v>
       </c>
       <c r="BL79" s="47">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM79" s="48" t="str">
@@ -18022,7 +18483,7 @@
         <v>51.660000000000082</v>
       </c>
       <c r="AS80" s="41">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-51.660000000000082</v>
       </c>
       <c r="AT80" s="41">
@@ -18071,11 +18532,11 @@
         <v>1505</v>
       </c>
       <c r="BI80" s="14" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ80" s="14" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ80" s="14" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK80" s="14">
@@ -18083,7 +18544,7 @@
         <v>0</v>
       </c>
       <c r="BL80" s="14">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM80" s="36" t="str">
@@ -18165,6 +18626,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -18387,34 +18875,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18431,29 +18917,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
MR24-045 day 11 model run
</commit_message>
<xml_diff>
--- a/data/mr24-045-experiment/MR24-045-MasterDataTable.xlsx
+++ b/data/mr24-045-experiment/MR24-045-MasterDataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/MR24-045-MPC-3L/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1470" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{970C3D87-E5E3-4C81-A6EA-E66F76EC7286}"/>
+  <xr:revisionPtr revIDLastSave="1624" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D091B6-3F2B-4BC1-A245-7155FD4BA60A}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1575" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="90">
   <si>
     <t>Batch Data</t>
   </si>
@@ -307,6 +307,9 @@
   <si>
     <t>MR24-045-806</t>
   </si>
+  <si>
+    <t>Antifoam totalizer reset due to schedule restart</t>
+  </si>
 </sst>
 </file>
 
@@ -318,7 +321,7 @@
     <numFmt numFmtId="166" formatCode="0.00000"/>
     <numFmt numFmtId="167" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -510,6 +513,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -990,7 +1000,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1077,6 +1087,9 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1229,6 +1242,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1546,91 +1563,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:71" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="68" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="69" t="s">
+      <c r="A1" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-      <c r="Z1" s="70"/>
-      <c r="AA1" s="70"/>
-      <c r="AB1" s="70"/>
-      <c r="AC1" s="70"/>
-      <c r="AD1" s="71"/>
-      <c r="AE1" s="84" t="s">
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="73"/>
+      <c r="W1" s="73"/>
+      <c r="X1" s="73"/>
+      <c r="Y1" s="73"/>
+      <c r="Z1" s="73"/>
+      <c r="AA1" s="73"/>
+      <c r="AB1" s="73"/>
+      <c r="AC1" s="73"/>
+      <c r="AD1" s="74"/>
+      <c r="AE1" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="AF1" s="85"/>
-      <c r="AG1" s="85"/>
-      <c r="AH1" s="85"/>
-      <c r="AI1" s="85"/>
-      <c r="AJ1" s="85"/>
-      <c r="AK1" s="85"/>
-      <c r="AL1" s="85"/>
-      <c r="AM1" s="85"/>
-      <c r="AN1" s="85"/>
-      <c r="AO1" s="85"/>
-      <c r="AP1" s="85"/>
-      <c r="AQ1" s="85"/>
-      <c r="AR1" s="85"/>
-      <c r="AS1" s="85"/>
-      <c r="AT1" s="85"/>
-      <c r="AU1" s="85"/>
-      <c r="AV1" s="85"/>
-      <c r="AW1" s="86"/>
-      <c r="AX1" s="78" t="s">
+      <c r="AF1" s="88"/>
+      <c r="AG1" s="88"/>
+      <c r="AH1" s="88"/>
+      <c r="AI1" s="88"/>
+      <c r="AJ1" s="88"/>
+      <c r="AK1" s="88"/>
+      <c r="AL1" s="88"/>
+      <c r="AM1" s="88"/>
+      <c r="AN1" s="88"/>
+      <c r="AO1" s="88"/>
+      <c r="AP1" s="88"/>
+      <c r="AQ1" s="88"/>
+      <c r="AR1" s="88"/>
+      <c r="AS1" s="88"/>
+      <c r="AT1" s="88"/>
+      <c r="AU1" s="88"/>
+      <c r="AV1" s="88"/>
+      <c r="AW1" s="89"/>
+      <c r="AX1" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="AY1" s="79"/>
-      <c r="AZ1" s="79"/>
-      <c r="BA1" s="79"/>
-      <c r="BB1" s="80"/>
-      <c r="BC1" s="81" t="s">
+      <c r="AY1" s="82"/>
+      <c r="AZ1" s="82"/>
+      <c r="BA1" s="82"/>
+      <c r="BB1" s="83"/>
+      <c r="BC1" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="BD1" s="82"/>
-      <c r="BE1" s="83"/>
-      <c r="BF1" s="75" t="s">
+      <c r="BD1" s="85"/>
+      <c r="BE1" s="86"/>
+      <c r="BF1" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="BG1" s="76"/>
-      <c r="BH1" s="76"/>
-      <c r="BI1" s="76"/>
-      <c r="BJ1" s="76"/>
-      <c r="BK1" s="76"/>
-      <c r="BL1" s="76"/>
-      <c r="BM1" s="76"/>
-      <c r="BN1" s="76"/>
-      <c r="BO1" s="76"/>
-      <c r="BP1" s="77"/>
-      <c r="BQ1" s="72" t="s">
+      <c r="BG1" s="79"/>
+      <c r="BH1" s="79"/>
+      <c r="BI1" s="79"/>
+      <c r="BJ1" s="79"/>
+      <c r="BK1" s="79"/>
+      <c r="BL1" s="79"/>
+      <c r="BM1" s="79"/>
+      <c r="BN1" s="79"/>
+      <c r="BO1" s="79"/>
+      <c r="BP1" s="80"/>
+      <c r="BQ1" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="BR1" s="73"/>
-      <c r="BS1" s="74"/>
+      <c r="BR1" s="76"/>
+      <c r="BS1" s="77"/>
     </row>
     <row r="2" spans="1:71" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
@@ -9172,7 +9189,7 @@
         <v>84.700000000000045</v>
       </c>
       <c r="AS35" s="45">
-        <f t="shared" ref="AS35:AS66" si="60">AQ35-AR35</f>
+        <f t="shared" ref="AS35:AS65" si="60">AQ35-AR35</f>
         <v>1755.3</v>
       </c>
       <c r="AT35" s="45">
@@ -12650,7 +12667,9 @@
       <c r="D51" s="3">
         <v>8</v>
       </c>
-      <c r="E51" s="3"/>
+      <c r="E51" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="F51" s="60">
         <v>45541.409976851901</v>
       </c>
@@ -12744,7 +12763,7 @@
       <c r="AK51" s="44">
         <v>33.090000000000003</v>
       </c>
-      <c r="AL51" s="6">
+      <c r="AL51" s="68">
         <v>5.29</v>
       </c>
       <c r="AM51" s="42">
@@ -12877,6 +12896,9 @@
       <c r="D52">
         <v>8</v>
       </c>
+      <c r="E52" t="s">
+        <v>89</v>
+      </c>
       <c r="F52" s="61">
         <v>45541.414027777799</v>
       </c>
@@ -12970,7 +12992,7 @@
       <c r="AK52" s="44">
         <v>26.68</v>
       </c>
-      <c r="AL52" s="44">
+      <c r="AL52" s="69">
         <v>3</v>
       </c>
       <c r="AM52" s="45">
@@ -13103,6 +13125,9 @@
       <c r="D53">
         <v>8</v>
       </c>
+      <c r="E53" t="s">
+        <v>89</v>
+      </c>
       <c r="F53" s="61">
         <v>45541.418136574102</v>
       </c>
@@ -13196,7 +13221,7 @@
       <c r="AK53" s="44">
         <v>1.24</v>
       </c>
-      <c r="AL53" s="44">
+      <c r="AL53" s="69">
         <v>6.66</v>
       </c>
       <c r="AM53" s="45">
@@ -13329,6 +13354,9 @@
       <c r="D54">
         <v>8</v>
       </c>
+      <c r="E54" t="s">
+        <v>89</v>
+      </c>
       <c r="F54" s="61">
         <v>45541.4217361111</v>
       </c>
@@ -13420,7 +13448,7 @@
       <c r="AK54" s="44">
         <v>10.53</v>
       </c>
-      <c r="AL54" s="44">
+      <c r="AL54" s="69">
         <v>6.76</v>
       </c>
       <c r="AM54" s="45">
@@ -13550,6 +13578,9 @@
       <c r="D55">
         <v>8</v>
       </c>
+      <c r="E55" t="s">
+        <v>89</v>
+      </c>
       <c r="F55" s="61">
         <v>45541.425601851901</v>
       </c>
@@ -13641,7 +13672,7 @@
       <c r="AK55" s="44">
         <v>7.31</v>
       </c>
-      <c r="AL55" s="44">
+      <c r="AL55" s="69">
         <v>6.44</v>
       </c>
       <c r="AM55" s="45">
@@ -13771,7 +13802,9 @@
       <c r="D56" s="5">
         <v>8</v>
       </c>
-      <c r="E56" s="5"/>
+      <c r="E56" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="F56" s="62">
         <v>45541.429097222201</v>
       </c>
@@ -13865,7 +13898,7 @@
       <c r="AK56" s="7">
         <v>28.23</v>
       </c>
-      <c r="AL56" s="7">
+      <c r="AL56" s="70">
         <v>6.52</v>
       </c>
       <c r="AM56" s="41">
@@ -13997,7 +14030,9 @@
         <v>9</v>
       </c>
       <c r="E57" s="3"/>
-      <c r="F57" s="60"/>
+      <c r="F57" s="60">
+        <v>45542.536215277803</v>
+      </c>
       <c r="G57" s="3">
         <v>4805.7299999999996</v>
       </c>
@@ -14094,7 +14129,7 @@
       </c>
       <c r="AM57" s="42">
         <f>BR57</f>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="AN57" s="6">
         <v>150.99</v>
@@ -14146,8 +14181,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC57" s="8"/>
-      <c r="BD57" s="9"/>
-      <c r="BE57" s="21"/>
+      <c r="BD57" s="46">
+        <f>BM57*24*60/BH57</f>
+        <v>1.2227344977136538E-2</v>
+      </c>
+      <c r="BE57" s="22">
+        <f>BP57/BH57</f>
+        <v>9.9999999999999995E-8</v>
+      </c>
       <c r="BF57" s="8">
         <f t="shared" si="17"/>
         <v>1.1345033880000001E-2</v>
@@ -14170,15 +14211,14 @@
       </c>
       <c r="BK57" s="10">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>22.446544179298034</v>
       </c>
       <c r="BL57" s="10" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM57" s="10">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="BN57" s="35" t="str">
         <f t="shared" si="32"/>
@@ -14189,20 +14229,19 @@
         <v/>
       </c>
       <c r="BP57" s="50">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>1.8357660000000001E-4</v>
       </c>
       <c r="BQ57" s="27">
         <f>IF(BL57&lt;&gt;"",BL57/0.000385,IF(BM57&lt;&gt;"",BM57/0.000385,BN57/0.000385))</f>
-        <v>0</v>
+        <v>40.487994551403375</v>
       </c>
       <c r="BR57" s="37">
         <f>IF(BL57&lt;&gt;"",BL57,IF(BM57&lt;&gt;"",BM57,BN57))</f>
-        <v>0</v>
+        <v>1.55878779022903E-2</v>
       </c>
       <c r="BS57" s="32">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>1.8357660000000001E-4</v>
       </c>
     </row>
     <row r="58" spans="1:71" x14ac:dyDescent="0.3">
@@ -14218,7 +14257,9 @@
       <c r="D58">
         <v>9</v>
       </c>
-      <c r="F58" s="61"/>
+      <c r="F58" s="61">
+        <v>45542.542280092603</v>
+      </c>
       <c r="G58">
         <v>4805.7299999999996</v>
       </c>
@@ -14315,7 +14356,7 @@
       </c>
       <c r="AM58" s="45">
         <f t="shared" ref="AM58:AM62" si="75">BR58</f>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="AN58" s="44">
         <v>167.56</v>
@@ -14367,8 +14408,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC58" s="11"/>
-      <c r="BD58" s="46"/>
-      <c r="BE58" s="22"/>
+      <c r="BD58" s="46">
+        <f>BM58*24*60/BH58</f>
+        <v>1.1176787745194918E-2</v>
+      </c>
+      <c r="BE58" s="22">
+        <f>BP58/BH58</f>
+        <v>3.3316909083529549E-3</v>
+      </c>
       <c r="BF58" s="11">
         <f t="shared" si="17"/>
         <v>1.1502565799999998E-2</v>
@@ -14391,15 +14438,14 @@
       </c>
       <c r="BK58" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>20.504264190069886</v>
       </c>
       <c r="BL58" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM58" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="BN58" s="48" t="str">
         <f t="shared" si="32"/>
@@ -14410,20 +14456,19 @@
         <v/>
       </c>
       <c r="BP58" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>6.1121202390098297</v>
       </c>
       <c r="BQ58" s="28">
         <f t="shared" ref="BQ58:BQ62" si="76">IF(BL58&lt;&gt;"",BL58/0.000385,IF(BM58&lt;&gt;"",BM58/0.000385,BN58/0.000385))</f>
-        <v>0</v>
+        <v>36.984603517442082</v>
       </c>
       <c r="BR58" s="49">
         <f t="shared" ref="BR58:BR62" si="77">IF(BL58&lt;&gt;"",BL58,IF(BM58&lt;&gt;"",BM58,BN58))</f>
-        <v>0</v>
+        <v>1.4239072354215201E-2</v>
       </c>
       <c r="BS58" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>6.1121202390098297</v>
       </c>
     </row>
     <row r="59" spans="1:71" x14ac:dyDescent="0.3">
@@ -14439,7 +14484,9 @@
       <c r="D59">
         <v>9</v>
       </c>
-      <c r="F59" s="61"/>
+      <c r="F59" s="61">
+        <v>45542.544826388897</v>
+      </c>
       <c r="G59">
         <v>4805.7299999999996</v>
       </c>
@@ -14536,7 +14583,7 @@
       </c>
       <c r="AM59" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="AN59" s="44">
         <v>211.31</v>
@@ -14588,8 +14635,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC59" s="11"/>
-      <c r="BD59" s="46"/>
-      <c r="BE59" s="22"/>
+      <c r="BD59" s="46">
+        <f>BM59*24*60/BH59</f>
+        <v>2.3999999999999973E-2</v>
+      </c>
+      <c r="BE59" s="22">
+        <f>BP59/BH59</f>
+        <v>4.1250564909925723E-3</v>
+      </c>
       <c r="BF59" s="11">
         <f t="shared" si="17"/>
         <v>9.8997816750000002E-3</v>
@@ -14612,15 +14665,14 @@
       </c>
       <c r="BK59" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>45.256144799999952</v>
       </c>
       <c r="BL59" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM59" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="BN59" s="48" t="str">
         <f t="shared" si="32"/>
@@ -14631,20 +14683,19 @@
         <v/>
       </c>
       <c r="BP59" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>7.77850641102249</v>
       </c>
       <c r="BQ59" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>81.630852813852727</v>
       </c>
       <c r="BR59" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>3.1427878333333298E-2</v>
       </c>
       <c r="BS59" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>7.77850641102249</v>
       </c>
     </row>
     <row r="60" spans="1:71" x14ac:dyDescent="0.3">
@@ -14660,13 +14711,15 @@
       <c r="D60">
         <v>9</v>
       </c>
-      <c r="F60" s="61"/>
+      <c r="F60" s="61">
+        <v>45542.547604166699</v>
+      </c>
       <c r="G60">
         <v>4805.7299999999996</v>
       </c>
       <c r="H60" s="44"/>
       <c r="I60" s="44">
-        <v>4576.09</v>
+        <v>4576.0950000000003</v>
       </c>
       <c r="J60" s="44">
         <v>19.2</v>
@@ -14757,7 +14810,7 @@
       </c>
       <c r="AM60" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="AN60" s="44">
         <v>204.07</v>
@@ -14808,7 +14861,9 @@
       <c r="BB60" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC60" s="11"/>
+      <c r="BC60" s="11">
+        <v>1.7999999999999999E-2</v>
+      </c>
       <c r="BE60" s="22"/>
       <c r="BF60" s="11">
         <f t="shared" si="17"/>
@@ -14832,11 +14887,11 @@
       </c>
       <c r="BK60" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>33.966593999999986</v>
       </c>
       <c r="BL60" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="BM60" s="48" t="str">
         <f t="shared" si="31"/>
@@ -14856,11 +14911,11 @@
       </c>
       <c r="BQ60" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>61.267305194805189</v>
       </c>
       <c r="BR60" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>2.3587912499999995E-2</v>
       </c>
       <c r="BS60" s="30">
         <f t="shared" si="21"/>
@@ -14880,7 +14935,9 @@
       <c r="D61">
         <v>9</v>
       </c>
-      <c r="F61" s="61"/>
+      <c r="F61" s="61">
+        <v>45542.550289351901</v>
+      </c>
       <c r="G61">
         <v>4805.7299999999996</v>
       </c>
@@ -14975,7 +15032,7 @@
       </c>
       <c r="AM61" s="45">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="AN61" s="44">
         <v>227.05</v>
@@ -15026,7 +15083,9 @@
       <c r="BB61" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC61" s="11"/>
+      <c r="BC61" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BE61" s="22"/>
       <c r="BF61" s="11">
         <f t="shared" si="17"/>
@@ -15050,11 +15109,11 @@
       </c>
       <c r="BK61" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>39.638652000000008</v>
       </c>
       <c r="BL61" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="BM61" s="48" t="str">
         <f t="shared" si="31"/>
@@ -15074,11 +15133,11 @@
       </c>
       <c r="BQ61" s="28">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>71.498290043290055</v>
       </c>
       <c r="BR61" s="49">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>2.752684166666667E-2</v>
       </c>
       <c r="BS61" s="30">
         <f t="shared" si="21"/>
@@ -15099,7 +15158,9 @@
         <v>9</v>
       </c>
       <c r="E62" s="5"/>
-      <c r="F62" s="62"/>
+      <c r="F62" s="62">
+        <v>45542.552824074097</v>
+      </c>
       <c r="G62" s="5">
         <v>4805.7299999999996</v>
       </c>
@@ -15196,7 +15257,7 @@
       </c>
       <c r="AM62" s="41">
         <f t="shared" si="75"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="AN62" s="7">
         <v>187.96</v>
@@ -15247,7 +15308,9 @@
       <c r="BB62" s="23">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC62" s="12"/>
+      <c r="BC62" s="12">
+        <v>8.5000000000000006E-3</v>
+      </c>
       <c r="BD62" s="5"/>
       <c r="BE62" s="23"/>
       <c r="BF62" s="12">
@@ -15272,11 +15335,11 @@
       </c>
       <c r="BK62" s="14">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>15.886534000000001</v>
       </c>
       <c r="BL62" s="14">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="BM62" s="48" t="str">
         <f t="shared" si="31"/>
@@ -15296,11 +15359,11 @@
       </c>
       <c r="BQ62" s="29">
         <f t="shared" si="76"/>
-        <v>0</v>
+        <v>28.655364357864364</v>
       </c>
       <c r="BR62" s="38">
         <f t="shared" si="77"/>
-        <v>0</v>
+        <v>1.1032315277777779E-2</v>
       </c>
       <c r="BS62" s="31">
         <f t="shared" si="21"/>
@@ -15321,70 +15384,137 @@
         <v>10</v>
       </c>
       <c r="E63" s="3"/>
-      <c r="F63" s="60"/>
+      <c r="F63" s="60">
+        <v>45543.405208333301</v>
+      </c>
       <c r="G63" s="63">
         <v>5497.99</v>
       </c>
       <c r="H63" s="6"/>
-      <c r="I63" s="6"/>
-      <c r="J63" s="6"/>
-      <c r="K63" s="6"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="6"/>
-      <c r="N63" s="6"/>
-      <c r="O63" s="6"/>
-      <c r="P63" s="6"/>
-      <c r="Q63" s="6"/>
+      <c r="I63" s="6">
+        <v>5803.62</v>
+      </c>
+      <c r="J63" s="6">
+        <v>20.399999999999999</v>
+      </c>
+      <c r="K63" s="6">
+        <v>18.7</v>
+      </c>
+      <c r="L63" s="6">
+        <v>91.5</v>
+      </c>
+      <c r="M63" s="6">
+        <v>17.3</v>
+      </c>
+      <c r="N63" s="6">
+        <v>347</v>
+      </c>
+      <c r="O63" s="6">
+        <v>1.72</v>
+      </c>
+      <c r="P63" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="Q63" s="6">
+        <v>1.64</v>
+      </c>
       <c r="R63" s="6"/>
-      <c r="S63" s="6"/>
-      <c r="T63" s="6"/>
-      <c r="U63" s="6"/>
-      <c r="V63" s="6"/>
-      <c r="W63" s="6"/>
-      <c r="X63" s="6"/>
-      <c r="Y63" s="6"/>
-      <c r="Z63" s="6"/>
-      <c r="AA63" s="6"/>
-      <c r="AB63" s="6"/>
-      <c r="AC63" s="6"/>
-      <c r="AD63" s="16"/>
-      <c r="AE63" s="6"/>
-      <c r="AF63" s="6"/>
-      <c r="AG63" s="6"/>
+      <c r="S63" s="6">
+        <v>0.11</v>
+      </c>
+      <c r="T63" s="6">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="U63" s="6">
+        <v>0.16</v>
+      </c>
+      <c r="V63" s="6">
+        <v>7.2460000000000004</v>
+      </c>
+      <c r="W63" s="6">
+        <v>95.9</v>
+      </c>
+      <c r="X63" s="6">
+        <v>11.5</v>
+      </c>
+      <c r="Y63" s="6">
+        <v>2.23</v>
+      </c>
+      <c r="Z63" s="6">
+        <v>146.4</v>
+      </c>
+      <c r="AA63" s="6">
+        <v>40.6</v>
+      </c>
+      <c r="AB63" s="6">
+        <v>84.1</v>
+      </c>
+      <c r="AC63" s="6">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="AD63" s="16">
+        <v>7.2869999999999999</v>
+      </c>
+      <c r="AE63" s="6">
+        <v>300</v>
+      </c>
+      <c r="AF63" s="6">
+        <v>47.8</v>
+      </c>
+      <c r="AG63" s="6">
+        <v>7.29</v>
+      </c>
       <c r="AH63" s="40">
         <f>AF63/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI63" s="6"/>
-      <c r="AJ63" s="6"/>
-      <c r="AK63" s="44"/>
-      <c r="AL63" s="6"/>
+        <v>0.47799999999999998</v>
+      </c>
+      <c r="AI63" s="6">
+        <v>34</v>
+      </c>
+      <c r="AJ63" s="6">
+        <v>22.065000000000001</v>
+      </c>
+      <c r="AK63" s="44">
+        <v>44.018999999999998</v>
+      </c>
+      <c r="AL63" s="6">
+        <f>AL51+1.91</f>
+        <v>7.2</v>
+      </c>
       <c r="AM63" s="42">
         <f>BR63</f>
-        <v>0</v>
-      </c>
-      <c r="AN63" s="6"/>
-      <c r="AO63" s="6"/>
-      <c r="AP63" s="6"/>
-      <c r="AQ63" s="6"/>
+        <v>5.1207888888888803E-3</v>
+      </c>
+      <c r="AN63" s="6">
+        <v>169.89</v>
+      </c>
+      <c r="AO63" s="6">
+        <v>65.31</v>
+      </c>
+      <c r="AP63" s="6">
+        <v>497</v>
+      </c>
+      <c r="AQ63" s="6">
+        <v>1984</v>
+      </c>
       <c r="AR63" s="40">
         <v>137.11999999999989</v>
       </c>
       <c r="AS63" s="40">
         <f t="shared" si="60"/>
-        <v>-137.11999999999989</v>
+        <v>1846.88</v>
       </c>
       <c r="AT63" s="40">
         <f t="shared" si="36"/>
-        <v>-150.99</v>
+        <v>18.899999999999977</v>
       </c>
       <c r="AU63" s="40">
         <f t="shared" si="37"/>
-        <v>-65.31</v>
+        <v>0</v>
       </c>
       <c r="AV63" s="40">
         <f t="shared" si="65"/>
-        <v>518</v>
+        <v>21</v>
       </c>
       <c r="AW63" s="24">
         <v>15</v>
@@ -15405,39 +15535,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC63" s="8"/>
-      <c r="BD63" s="9"/>
-      <c r="BE63" s="21"/>
+      <c r="BD63" s="46">
+        <f>BM63*24*60/BH63</f>
+        <v>3.999999999999994E-3</v>
+      </c>
+      <c r="BE63" s="22">
+        <f>BP63/BH63</f>
+        <v>3.9797979551218672E-3</v>
+      </c>
       <c r="BF63" s="8">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.0341945239999999E-2</v>
       </c>
       <c r="BG63" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.892401145599999</v>
       </c>
       <c r="BH63" s="9">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI63" s="10" t="str">
+        <v>1843.4839999999999</v>
+      </c>
+      <c r="BI63" s="10">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ63" s="10" t="str">
+        <v>9.2157024416810771E-2</v>
+      </c>
+      <c r="BJ63" s="10">
         <f t="shared" si="9"/>
-        <v/>
+        <v>9.9935294117647053E-2</v>
       </c>
       <c r="BK63" s="10">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>7.3739359999999881</v>
       </c>
       <c r="BL63" s="10" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM63" s="10">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>5.1207888888888803E-3</v>
       </c>
       <c r="BN63" s="35" t="str">
         <f t="shared" si="32"/>
@@ -15448,20 +15583,19 @@
         <v/>
       </c>
       <c r="BP63" s="50">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>7.33669385349988</v>
       </c>
       <c r="BQ63" s="27">
         <f>IF(BL63&lt;&gt;"",BL63/0.000385,IF(BM63&lt;&gt;"",BM63/0.000385,BN63/0.000385))</f>
-        <v>0</v>
+        <v>13.300750360750339</v>
       </c>
       <c r="BR63" s="37">
         <f>IF(BL63&lt;&gt;"",BL63,IF(BM63&lt;&gt;"",BM63,BN63))</f>
-        <v>0</v>
+        <v>5.1207888888888803E-3</v>
       </c>
       <c r="BS63" s="32">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>7.33669385349988</v>
       </c>
     </row>
     <row r="64" spans="1:71" x14ac:dyDescent="0.3">
@@ -15477,70 +15611,137 @@
       <c r="D64">
         <v>10</v>
       </c>
-      <c r="F64" s="61"/>
+      <c r="F64" s="61">
+        <v>45543.413275462997</v>
+      </c>
       <c r="G64" s="64">
         <v>5497.99</v>
       </c>
       <c r="H64" s="44"/>
-      <c r="I64" s="44"/>
-      <c r="J64" s="44"/>
-      <c r="K64" s="44"/>
-      <c r="L64" s="44"/>
-      <c r="M64" s="44"/>
-      <c r="N64" s="44"/>
-      <c r="O64" s="44"/>
-      <c r="P64" s="44"/>
-      <c r="Q64" s="44"/>
+      <c r="I64" s="44">
+        <v>5945.67</v>
+      </c>
+      <c r="J64" s="44">
+        <v>20.6</v>
+      </c>
+      <c r="K64" s="44">
+        <v>19.3</v>
+      </c>
+      <c r="L64" s="44">
+        <v>93.9</v>
+      </c>
+      <c r="M64" s="44">
+        <v>17.8</v>
+      </c>
+      <c r="N64" s="44">
+        <v>348</v>
+      </c>
+      <c r="O64" s="44">
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="P64" s="44">
+        <v>0.21</v>
+      </c>
+      <c r="Q64" s="44">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="R64" s="44"/>
-      <c r="S64" s="44"/>
-      <c r="T64" s="44"/>
-      <c r="U64" s="44"/>
-      <c r="V64" s="44"/>
-      <c r="W64" s="44"/>
-      <c r="X64" s="44"/>
-      <c r="Y64" s="44"/>
-      <c r="Z64" s="44"/>
-      <c r="AA64" s="44"/>
-      <c r="AB64" s="44"/>
-      <c r="AC64" s="44"/>
-      <c r="AD64" s="17"/>
-      <c r="AE64" s="44"/>
-      <c r="AF64" s="44"/>
-      <c r="AG64" s="44"/>
+      <c r="S64" s="44">
+        <v>0.1</v>
+      </c>
+      <c r="T64" s="44">
+        <v>0.15</v>
+      </c>
+      <c r="U64" s="44">
+        <v>0.16</v>
+      </c>
+      <c r="V64" s="44">
+        <v>7.2619999999999996</v>
+      </c>
+      <c r="W64" s="44">
+        <v>105</v>
+      </c>
+      <c r="X64" s="44">
+        <v>55.7</v>
+      </c>
+      <c r="Y64" s="44">
+        <v>2.15</v>
+      </c>
+      <c r="Z64" s="44">
+        <v>154.19999999999999</v>
+      </c>
+      <c r="AA64" s="44">
+        <v>46.1</v>
+      </c>
+      <c r="AB64" s="44">
+        <v>92.1</v>
+      </c>
+      <c r="AC64" s="44">
+        <v>45.2</v>
+      </c>
+      <c r="AD64" s="17">
+        <v>7.3029999999999999</v>
+      </c>
+      <c r="AE64" s="44">
+        <v>300</v>
+      </c>
+      <c r="AF64" s="44">
+        <v>49.9</v>
+      </c>
+      <c r="AG64" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH64" s="45">
         <f t="shared" ref="AH64:AH68" si="78">AF64/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI64" s="44"/>
-      <c r="AJ64" s="44"/>
-      <c r="AK64" s="44"/>
-      <c r="AL64" s="44"/>
+        <v>0.499</v>
+      </c>
+      <c r="AI64" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ64" s="44">
+        <v>24.568000000000001</v>
+      </c>
+      <c r="AK64" s="44">
+        <v>27.469000000000001</v>
+      </c>
+      <c r="AL64" s="44">
+        <f>AL52+1.86</f>
+        <v>4.8600000000000003</v>
+      </c>
       <c r="AM64" s="45">
         <f t="shared" ref="AM64:AM68" si="79">BR64</f>
-        <v>0</v>
-      </c>
-      <c r="AN64" s="44"/>
-      <c r="AO64" s="44"/>
-      <c r="AP64" s="44"/>
-      <c r="AQ64" s="44"/>
+        <v>1.1401776999282799E-2</v>
+      </c>
+      <c r="AN64" s="44">
+        <v>185.31</v>
+      </c>
+      <c r="AO64" s="44">
+        <v>68.25</v>
+      </c>
+      <c r="AP64" s="44">
+        <v>481</v>
+      </c>
+      <c r="AQ64" s="44">
+        <v>1988</v>
+      </c>
       <c r="AR64" s="45">
         <v>45.769999999999982</v>
       </c>
       <c r="AS64" s="45">
         <f t="shared" si="60"/>
-        <v>-45.769999999999982</v>
+        <v>1942.23</v>
       </c>
       <c r="AT64" s="45">
         <f t="shared" si="36"/>
-        <v>-167.56</v>
+        <v>17.75</v>
       </c>
       <c r="AU64" s="45">
         <f t="shared" si="37"/>
-        <v>-61.42</v>
+        <v>6.8299999999999983</v>
       </c>
       <c r="AV64" s="45">
         <f t="shared" si="65"/>
-        <v>501</v>
+        <v>20</v>
       </c>
       <c r="AW64" s="25">
         <v>15</v>
@@ -15561,39 +15762,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC64" s="11"/>
-      <c r="BD64" s="46"/>
-      <c r="BE64" s="22"/>
+      <c r="BD64" s="46">
+        <f>BM64*24*60/BH64</f>
+        <v>8.8967442096820649E-3</v>
+      </c>
+      <c r="BE64" s="22">
+        <f>BP64/BH64</f>
+        <v>5.5208033108114681E-3</v>
+      </c>
       <c r="BF64" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.068519603E-2</v>
       </c>
       <c r="BG64" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15.386682283200003</v>
       </c>
       <c r="BH64" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI64" s="47" t="str">
+        <v>1845.4569999999999</v>
+      </c>
+      <c r="BI64" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ64" s="47" t="str">
+        <v>0.10041415215851685</v>
+      </c>
+      <c r="BJ64" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.10900588235294117</v>
       </c>
       <c r="BK64" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>16.418558878967232</v>
       </c>
       <c r="BL64" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM64" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1.1401776999282799E-2</v>
       </c>
       <c r="BN64" s="48" t="str">
         <f t="shared" si="32"/>
@@ -15604,20 +15810,19 @@
         <v/>
       </c>
       <c r="BP64" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>10.188405115560199</v>
       </c>
       <c r="BQ64" s="28">
         <f t="shared" ref="BQ64:BQ68" si="80">IF(BL64&lt;&gt;"",BL64/0.000385,IF(BM64&lt;&gt;"",BM64/0.000385,BN64/0.000385))</f>
-        <v>0</v>
+        <v>29.615005192942338</v>
       </c>
       <c r="BR64" s="49">
         <f t="shared" ref="BR64:BR68" si="81">IF(BL64&lt;&gt;"",BL64,IF(BM64&lt;&gt;"",BM64,BN64))</f>
-        <v>0</v>
+        <v>1.1401776999282799E-2</v>
       </c>
       <c r="BS64" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>10.188405115560199</v>
       </c>
     </row>
     <row r="65" spans="1:71" x14ac:dyDescent="0.3">
@@ -15633,70 +15838,137 @@
       <c r="D65">
         <v>10</v>
       </c>
-      <c r="F65" s="61"/>
+      <c r="F65" s="61">
+        <v>45543.423032407401</v>
+      </c>
       <c r="G65" s="64">
         <v>5497.99</v>
       </c>
       <c r="H65" s="44"/>
-      <c r="I65" s="44"/>
-      <c r="J65" s="44"/>
-      <c r="K65" s="44"/>
-      <c r="L65" s="44"/>
-      <c r="M65" s="44"/>
-      <c r="N65" s="44"/>
-      <c r="O65" s="44"/>
-      <c r="P65" s="44"/>
-      <c r="Q65" s="44"/>
+      <c r="I65" s="44">
+        <v>5235.63</v>
+      </c>
+      <c r="J65" s="44">
+        <v>20.2</v>
+      </c>
+      <c r="K65" s="44">
+        <v>18</v>
+      </c>
+      <c r="L65" s="44">
+        <v>89.1</v>
+      </c>
+      <c r="M65" s="44">
+        <v>19.2</v>
+      </c>
+      <c r="N65" s="44">
+        <v>438</v>
+      </c>
+      <c r="O65" s="44">
+        <v>2.36</v>
+      </c>
+      <c r="P65" s="44">
+        <v>0.22</v>
+      </c>
+      <c r="Q65" s="44">
+        <v>3.22</v>
+      </c>
       <c r="R65" s="44"/>
-      <c r="S65" s="44"/>
-      <c r="T65" s="44"/>
-      <c r="U65" s="44"/>
-      <c r="V65" s="44"/>
-      <c r="W65" s="44"/>
-      <c r="X65" s="44"/>
-      <c r="Y65" s="44"/>
-      <c r="Z65" s="44"/>
-      <c r="AA65" s="44"/>
-      <c r="AB65" s="44"/>
-      <c r="AC65" s="44"/>
-      <c r="AD65" s="17"/>
-      <c r="AE65" s="44"/>
-      <c r="AF65" s="44"/>
-      <c r="AG65" s="44"/>
+      <c r="S65" s="44">
+        <v>0.78</v>
+      </c>
+      <c r="T65" s="44">
+        <v>2.21</v>
+      </c>
+      <c r="U65" s="44">
+        <v>2.19</v>
+      </c>
+      <c r="V65" s="44">
+        <v>7.2469999999999999</v>
+      </c>
+      <c r="W65" s="44">
+        <v>118.5</v>
+      </c>
+      <c r="X65" s="44">
+        <v>46.8</v>
+      </c>
+      <c r="Y65" s="44">
+        <v>1.5</v>
+      </c>
+      <c r="Z65" s="44">
+        <v>176.3</v>
+      </c>
+      <c r="AA65" s="44">
+        <v>50.2</v>
+      </c>
+      <c r="AB65" s="44">
+        <v>104</v>
+      </c>
+      <c r="AC65" s="44">
+        <v>37.9</v>
+      </c>
+      <c r="AD65" s="17">
+        <v>7.2880000000000003</v>
+      </c>
+      <c r="AE65" s="44">
+        <v>298</v>
+      </c>
+      <c r="AF65" s="44">
+        <v>50.4</v>
+      </c>
+      <c r="AG65" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH65" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI65" s="44"/>
-      <c r="AJ65" s="44"/>
-      <c r="AK65" s="44"/>
-      <c r="AL65" s="44"/>
+        <v>0.504</v>
+      </c>
+      <c r="AI65" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ65" s="44">
+        <v>38.045999999999999</v>
+      </c>
+      <c r="AK65" s="44">
+        <v>5.1144999999999996</v>
+      </c>
+      <c r="AL65" s="44">
+        <f>AL53+1.87</f>
+        <v>8.5300000000000011</v>
+      </c>
       <c r="AM65" s="45">
         <f t="shared" si="79"/>
-        <v>0</v>
-      </c>
-      <c r="AN65" s="44"/>
-      <c r="AO65" s="44"/>
-      <c r="AP65" s="44"/>
-      <c r="AQ65" s="44"/>
+        <v>2.08588154275034E-2</v>
+      </c>
+      <c r="AN65" s="44">
+        <v>249.44</v>
+      </c>
+      <c r="AO65" s="44">
+        <v>84.76</v>
+      </c>
+      <c r="AP65" s="44">
+        <v>384</v>
+      </c>
+      <c r="AQ65" s="44">
+        <v>2061</v>
+      </c>
       <c r="AR65" s="45">
         <v>84.700000000000045</v>
       </c>
       <c r="AS65" s="45">
         <f t="shared" si="60"/>
-        <v>-84.700000000000045</v>
+        <v>1976.3</v>
       </c>
       <c r="AT65" s="45">
         <f t="shared" si="36"/>
-        <v>-211.31</v>
+        <v>38.129999999999995</v>
       </c>
       <c r="AU65" s="45">
         <f t="shared" si="37"/>
-        <v>-76.27</v>
+        <v>8.4900000000000091</v>
       </c>
       <c r="AV65" s="45">
         <f t="shared" si="65"/>
-        <v>430</v>
+        <v>46</v>
       </c>
       <c r="AW65" s="25">
         <v>15</v>
@@ -15717,39 +15989,44 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC65" s="11"/>
-      <c r="BD65" s="46"/>
-      <c r="BE65" s="22"/>
+      <c r="BD65" s="46">
+        <f>BM65*24*60/BH65</f>
+        <v>1.5636859162771067E-2</v>
+      </c>
+      <c r="BE65" s="22">
+        <f>BP65/BH65</f>
+        <v>1.6524849493275854E-3</v>
+      </c>
       <c r="BF65" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.0372808699999998E-2</v>
       </c>
       <c r="BG65" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.936844527999996</v>
       </c>
       <c r="BH65" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI65" s="47" t="str">
+        <v>1920.8905</v>
+      </c>
+      <c r="BI65" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ65" s="47" t="str">
+        <v>0.12985643897973362</v>
+      </c>
+      <c r="BJ65" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.14672941176470589</v>
       </c>
       <c r="BK65" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>30.036694215604896</v>
       </c>
       <c r="BL65" s="47" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
       <c r="BM65" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
+        <v>2.08588154275034E-2</v>
       </c>
       <c r="BN65" s="48" t="str">
         <f t="shared" si="32"/>
@@ -15760,20 +16037,19 @@
         <v/>
       </c>
       <c r="BP65" s="51">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>3.17424264055634</v>
       </c>
       <c r="BQ65" s="28">
         <f t="shared" si="80"/>
-        <v>0</v>
+        <v>54.178741370138702</v>
       </c>
       <c r="BR65" s="49">
         <f t="shared" si="81"/>
-        <v>0</v>
+        <v>2.08588154275034E-2</v>
       </c>
       <c r="BS65" s="30">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>3.17424264055634</v>
       </c>
     </row>
     <row r="66" spans="1:71" x14ac:dyDescent="0.3">
@@ -15789,70 +16065,137 @@
       <c r="D66">
         <v>10</v>
       </c>
-      <c r="F66" s="61"/>
+      <c r="F66" s="61">
+        <v>45543.425671296303</v>
+      </c>
       <c r="G66" s="64">
         <v>5497.99</v>
       </c>
       <c r="H66" s="44"/>
-      <c r="I66" s="44"/>
-      <c r="J66" s="44"/>
-      <c r="K66" s="44"/>
-      <c r="L66" s="44"/>
-      <c r="M66" s="44"/>
-      <c r="N66" s="44"/>
-      <c r="O66" s="44"/>
-      <c r="P66" s="44"/>
-      <c r="Q66" s="44"/>
+      <c r="I66" s="44">
+        <v>5350.9049999999997</v>
+      </c>
+      <c r="J66" s="44">
+        <v>20.2</v>
+      </c>
+      <c r="K66" s="44">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="L66" s="44">
+        <v>89.7</v>
+      </c>
+      <c r="M66" s="44">
+        <v>19</v>
+      </c>
+      <c r="N66" s="44">
+        <v>430</v>
+      </c>
+      <c r="O66" s="44">
+        <v>1.71</v>
+      </c>
+      <c r="P66" s="44">
+        <v>0.21</v>
+      </c>
+      <c r="Q66" s="44">
+        <v>1.31</v>
+      </c>
       <c r="R66" s="44"/>
-      <c r="S66" s="44"/>
-      <c r="T66" s="44"/>
-      <c r="U66" s="44"/>
-      <c r="V66" s="44"/>
-      <c r="W66" s="44"/>
-      <c r="X66" s="44"/>
-      <c r="Y66" s="44"/>
-      <c r="Z66" s="44"/>
-      <c r="AA66" s="44"/>
-      <c r="AB66" s="44"/>
-      <c r="AC66" s="44"/>
-      <c r="AD66" s="17"/>
-      <c r="AE66" s="44"/>
-      <c r="AF66" s="44"/>
-      <c r="AG66" s="44"/>
+      <c r="S66" s="44">
+        <v>0.6</v>
+      </c>
+      <c r="T66" s="44">
+        <v>2.08</v>
+      </c>
+      <c r="U66" s="44">
+        <v>2.54</v>
+      </c>
+      <c r="V66" s="44">
+        <v>7.2779999999999996</v>
+      </c>
+      <c r="W66" s="44">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="X66" s="44">
+        <v>30</v>
+      </c>
+      <c r="Y66" s="44">
+        <v>1.48</v>
+      </c>
+      <c r="Z66" s="44">
+        <v>183.1</v>
+      </c>
+      <c r="AA66" s="44">
+        <v>58.4</v>
+      </c>
+      <c r="AB66" s="44">
+        <v>112.5</v>
+      </c>
+      <c r="AC66" s="44">
+        <v>24.3</v>
+      </c>
+      <c r="AD66" s="17">
+        <v>7.319</v>
+      </c>
+      <c r="AE66" s="44">
+        <v>301</v>
+      </c>
+      <c r="AF66" s="44">
+        <v>51.1</v>
+      </c>
+      <c r="AG66" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH66" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI66" s="44"/>
-      <c r="AJ66" s="44"/>
-      <c r="AK66" s="44"/>
-      <c r="AL66" s="44"/>
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="AI66" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ66" s="44">
+        <v>43.091000000000001</v>
+      </c>
+      <c r="AK66" s="44">
+        <v>13.548</v>
+      </c>
+      <c r="AL66" s="44">
+        <f>AL54+1.91</f>
+        <v>8.67</v>
+      </c>
       <c r="AM66" s="45">
         <f t="shared" si="79"/>
-        <v>0</v>
-      </c>
-      <c r="AN66" s="44"/>
-      <c r="AO66" s="44"/>
-      <c r="AP66" s="44"/>
-      <c r="AQ66" s="44"/>
+        <v>2.2755468611111111E-2</v>
+      </c>
+      <c r="AN66" s="44">
+        <v>233.93</v>
+      </c>
+      <c r="AO66" s="44">
+        <v>70.87</v>
+      </c>
+      <c r="AP66" s="44">
+        <v>406</v>
+      </c>
+      <c r="AQ66" s="44">
+        <v>2044</v>
+      </c>
       <c r="AR66" s="45">
         <v>47.420000000000073</v>
       </c>
       <c r="AS66" s="45">
-        <f t="shared" si="60"/>
-        <v>-47.420000000000073</v>
+        <f>AQ66-AR66</f>
+        <v>1996.58</v>
       </c>
       <c r="AT66" s="45">
         <f t="shared" si="36"/>
-        <v>-204.07</v>
+        <v>29.860000000000014</v>
       </c>
       <c r="AU66" s="45">
         <f t="shared" si="37"/>
-        <v>-70.87</v>
+        <v>0</v>
       </c>
       <c r="AV66" s="45">
         <f t="shared" si="65"/>
-        <v>443</v>
+        <v>37</v>
       </c>
       <c r="AW66" s="25">
         <v>15</v>
@@ -15872,35 +16215,37 @@
       <c r="BB66" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC66" s="11"/>
+      <c r="BC66" s="11">
+        <v>1.72E-2</v>
+      </c>
       <c r="BE66" s="22"/>
       <c r="BF66" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.034474187E-2</v>
       </c>
       <c r="BG66" s="46">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14.8964282928</v>
       </c>
       <c r="BH66" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI66" s="47" t="str">
+        <v>1905.1089999999999</v>
+      </c>
+      <c r="BI66" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ66" s="47" t="str">
+        <v>0.12279087443290647</v>
+      </c>
+      <c r="BJ66" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.13760588235294119</v>
       </c>
       <c r="BK66" s="47">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>32.767874800000001</v>
       </c>
       <c r="BL66" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.2755468611111111E-2</v>
       </c>
       <c r="BM66" s="48" t="str">
         <f t="shared" si="31"/>
@@ -15912,7 +16257,7 @@
       </c>
       <c r="BO66" s="47">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>8.0490855249999989</v>
       </c>
       <c r="BP66" s="51" t="str">
         <f t="shared" si="28"/>
@@ -15920,15 +16265,15 @@
       </c>
       <c r="BQ66" s="28">
         <f t="shared" si="80"/>
-        <v>0</v>
+        <v>59.105113275613277</v>
       </c>
       <c r="BR66" s="49">
         <f t="shared" si="81"/>
-        <v>0</v>
+        <v>2.2755468611111111E-2</v>
       </c>
       <c r="BS66" s="30">
         <f t="shared" si="21"/>
-        <v>11.512499999999999</v>
+        <v>8.0490855249999989</v>
       </c>
     </row>
     <row r="67" spans="1:71" x14ac:dyDescent="0.3">
@@ -15944,70 +16289,133 @@
       <c r="D67">
         <v>10</v>
       </c>
-      <c r="F67" s="61"/>
+      <c r="F67" s="61">
+        <v>45543.428912037001</v>
+      </c>
       <c r="G67" s="64">
         <v>5497.99</v>
       </c>
       <c r="H67" s="44"/>
-      <c r="I67" s="44"/>
-      <c r="J67" s="44"/>
-      <c r="K67" s="44"/>
-      <c r="L67" s="44"/>
-      <c r="M67" s="44"/>
-      <c r="N67" s="44"/>
+      <c r="I67" s="44">
+        <v>2975.5050000000001</v>
+      </c>
+      <c r="J67" s="44">
+        <v>21.1</v>
+      </c>
+      <c r="K67" s="44">
+        <v>8.32</v>
+      </c>
+      <c r="L67" s="44">
+        <v>39.5</v>
+      </c>
+      <c r="M67" s="44">
+        <v>15.6</v>
+      </c>
+      <c r="N67" s="44">
+        <v>818</v>
+      </c>
       <c r="O67" s="44"/>
-      <c r="P67" s="44"/>
-      <c r="Q67" s="44"/>
+      <c r="P67" s="44">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="Q67" s="44">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="R67" s="44"/>
-      <c r="S67" s="44"/>
-      <c r="T67" s="44"/>
+      <c r="S67" s="44">
+        <v>0.75</v>
+      </c>
+      <c r="T67" s="44">
+        <v>3.48</v>
+      </c>
       <c r="U67" s="44"/>
-      <c r="V67" s="44"/>
-      <c r="W67" s="44"/>
-      <c r="X67" s="44"/>
-      <c r="Y67" s="44"/>
-      <c r="Z67" s="44"/>
-      <c r="AA67" s="44"/>
-      <c r="AB67" s="44"/>
-      <c r="AC67" s="44"/>
-      <c r="AD67" s="17"/>
-      <c r="AE67" s="44"/>
-      <c r="AF67" s="44"/>
-      <c r="AG67" s="44"/>
+      <c r="V67" s="44">
+        <v>7.032</v>
+      </c>
+      <c r="W67" s="44">
+        <v>66.3</v>
+      </c>
+      <c r="X67" s="44">
+        <v>86</v>
+      </c>
+      <c r="Y67" s="44">
+        <v>7.2</v>
+      </c>
+      <c r="Z67" s="44">
+        <v>327.9</v>
+      </c>
+      <c r="AA67" s="44">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="AB67" s="44">
+        <v>58.1</v>
+      </c>
+      <c r="AC67" s="44">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="AD67" s="17">
+        <v>7.069</v>
+      </c>
+      <c r="AE67" s="44">
+        <v>301</v>
+      </c>
+      <c r="AF67" s="44">
+        <v>45.2</v>
+      </c>
+      <c r="AG67" s="44">
+        <v>7.09</v>
+      </c>
       <c r="AH67" s="45">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI67" s="44"/>
-      <c r="AJ67" s="44"/>
-      <c r="AK67" s="44"/>
-      <c r="AL67" s="44"/>
+        <v>0.45200000000000001</v>
+      </c>
+      <c r="AI67" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ67" s="44">
+        <v>157.88999999999999</v>
+      </c>
+      <c r="AK67" s="44">
+        <v>7.3125999999999998</v>
+      </c>
+      <c r="AL67" s="44">
+        <f>AL55+1.84</f>
+        <v>8.2800000000000011</v>
+      </c>
       <c r="AM67" s="45">
         <f t="shared" si="79"/>
-        <v>0</v>
-      </c>
-      <c r="AN67" s="44"/>
-      <c r="AO67" s="44"/>
-      <c r="AP67" s="44"/>
-      <c r="AQ67" s="44"/>
+        <v>2.8444202777777781E-2</v>
+      </c>
+      <c r="AN67" s="44">
+        <v>261.68</v>
+      </c>
+      <c r="AO67" s="44">
+        <v>77.819999999999993</v>
+      </c>
+      <c r="AP67" s="44">
+        <v>353</v>
+      </c>
+      <c r="AQ67" s="44">
+        <v>2185</v>
+      </c>
       <c r="AR67" s="45">
         <v>133.55999999999995</v>
       </c>
       <c r="AS67" s="45">
-        <f t="shared" ref="AS67:AS80" si="82">AQ67-AR67</f>
-        <v>-133.55999999999995</v>
+        <f>AQ67-AR67</f>
+        <v>2051.44</v>
       </c>
       <c r="AT67" s="45">
         <f t="shared" si="36"/>
-        <v>-227.05</v>
+        <v>34.629999999999995</v>
       </c>
       <c r="AU67" s="45">
         <f t="shared" si="37"/>
-        <v>-77.819999999999993</v>
+        <v>0</v>
       </c>
       <c r="AV67" s="45">
         <f t="shared" si="65"/>
-        <v>394</v>
+        <v>41</v>
       </c>
       <c r="AW67" s="25">
         <v>15</v>
@@ -16027,47 +16435,49 @@
       <c r="BB67" s="22">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC67" s="11"/>
+      <c r="BC67" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BE67" s="22"/>
       <c r="BF67" s="11">
-        <f t="shared" ref="BF67:BF74" si="83">BB67*K67*BH67/1000</f>
-        <v>0</v>
+        <f t="shared" ref="BF67:BF74" si="82">BB67*K67*BH67/1000</f>
+        <v>5.1117645696000013E-3</v>
       </c>
       <c r="BG67" s="46">
-        <f t="shared" ref="BG67:BG74" si="84">BF67*24*60</f>
-        <v>0</v>
+        <f t="shared" ref="BG67:BG74" si="83">BF67*24*60</f>
+        <v>7.3609409802240027</v>
       </c>
       <c r="BH67" s="46">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI67" s="47" t="str">
+        <v>2047.9826000000003</v>
+      </c>
+      <c r="BI67" s="47">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="BJ67" s="47" t="str">
+        <v>0.12777452308432696</v>
+      </c>
+      <c r="BJ67" s="47">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.1539294117647059</v>
       </c>
       <c r="BK67" s="47">
-        <f t="shared" ref="BK67:BK74" si="85">AM67*24*60</f>
-        <v>0</v>
+        <f t="shared" ref="BK67:BK74" si="84">AM67*24*60</f>
+        <v>40.959652000000006</v>
       </c>
       <c r="BL67" s="47">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2.8444202777777781E-2</v>
       </c>
       <c r="BM67" s="48" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="BN67" s="48" t="str">
-        <f t="shared" ref="BN67:BN74" si="86">IF(B67="No MPC", BB67*K67*BH67/1000,"")</f>
+        <f t="shared" ref="BN67:BN74" si="85">IF(B67="No MPC", BB67*K67*BH67/1000,"")</f>
         <v/>
       </c>
       <c r="BO67" s="47">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>15.001472545000004</v>
       </c>
       <c r="BP67" s="51" t="str">
         <f t="shared" si="28"/>
@@ -16075,15 +16485,15 @@
       </c>
       <c r="BQ67" s="28">
         <f t="shared" si="80"/>
-        <v>0</v>
+        <v>73.881046176046183</v>
       </c>
       <c r="BR67" s="49">
         <f t="shared" si="81"/>
-        <v>0</v>
+        <v>2.8444202777777781E-2</v>
       </c>
       <c r="BS67" s="30">
-        <f t="shared" ref="BS67:BS74" si="87">IF(BO67&lt;&gt;"",BO67,BP67)</f>
-        <v>11.512499999999999</v>
+        <f t="shared" ref="BS67:BS74" si="86">IF(BO67&lt;&gt;"",BO67,BP67)</f>
+        <v>15.001472545000004</v>
       </c>
     </row>
     <row r="68" spans="1:71" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -16100,70 +16510,137 @@
         <v>10</v>
       </c>
       <c r="E68" s="5"/>
-      <c r="F68" s="62"/>
+      <c r="F68" s="62">
+        <v>45543.4315740741</v>
+      </c>
       <c r="G68" s="65">
         <v>5497.99</v>
       </c>
       <c r="H68" s="7"/>
-      <c r="I68" s="7"/>
-      <c r="J68" s="7"/>
-      <c r="K68" s="7"/>
-      <c r="L68" s="7"/>
-      <c r="M68" s="7"/>
-      <c r="N68" s="7"/>
-      <c r="O68" s="7"/>
-      <c r="P68" s="7"/>
-      <c r="Q68" s="7"/>
+      <c r="I68" s="7">
+        <v>5979</v>
+      </c>
+      <c r="J68" s="7">
+        <v>21.5</v>
+      </c>
+      <c r="K68" s="7">
+        <v>19.7</v>
+      </c>
+      <c r="L68" s="7">
+        <v>92</v>
+      </c>
+      <c r="M68" s="7">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="N68" s="7">
+        <v>367</v>
+      </c>
+      <c r="O68" s="7">
+        <v>1.57</v>
+      </c>
+      <c r="P68" s="7">
+        <v>0.19</v>
+      </c>
+      <c r="Q68" s="7">
+        <v>0.66</v>
+      </c>
       <c r="R68" s="7"/>
-      <c r="S68" s="7"/>
-      <c r="T68" s="7"/>
-      <c r="U68" s="7"/>
-      <c r="V68" s="7"/>
-      <c r="W68" s="7"/>
-      <c r="X68" s="7"/>
-      <c r="Y68" s="7"/>
-      <c r="Z68" s="7"/>
-      <c r="AA68" s="7"/>
-      <c r="AB68" s="7"/>
-      <c r="AC68" s="7"/>
-      <c r="AD68" s="18"/>
-      <c r="AE68" s="7"/>
-      <c r="AF68" s="7"/>
-      <c r="AG68" s="7"/>
+      <c r="S68" s="7">
+        <v>0.17</v>
+      </c>
+      <c r="T68" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="U68" s="7">
+        <v>0.73</v>
+      </c>
+      <c r="V68" s="7">
+        <v>7.2640000000000002</v>
+      </c>
+      <c r="W68" s="7">
+        <v>120.2</v>
+      </c>
+      <c r="X68" s="7">
+        <v>31.7</v>
+      </c>
+      <c r="Y68" s="7">
+        <v>1.79</v>
+      </c>
+      <c r="Z68" s="7">
+        <v>160</v>
+      </c>
+      <c r="AA68" s="7">
+        <v>53</v>
+      </c>
+      <c r="AB68" s="7">
+        <v>105.4</v>
+      </c>
+      <c r="AC68" s="7">
+        <v>25.6</v>
+      </c>
+      <c r="AD68" s="18">
+        <v>7.3049999999999997</v>
+      </c>
+      <c r="AE68" s="7">
+        <v>299</v>
+      </c>
+      <c r="AF68" s="7">
+        <v>49.3</v>
+      </c>
+      <c r="AG68" s="7">
+        <v>7.3</v>
+      </c>
       <c r="AH68" s="41">
         <f t="shared" si="78"/>
-        <v>0</v>
-      </c>
-      <c r="AI68" s="7"/>
-      <c r="AJ68" s="7"/>
-      <c r="AK68" s="7"/>
-      <c r="AL68" s="7"/>
+        <v>0.49299999999999999</v>
+      </c>
+      <c r="AI68" s="7">
+        <v>34</v>
+      </c>
+      <c r="AJ68" s="7">
+        <v>28.271000000000001</v>
+      </c>
+      <c r="AK68" s="7">
+        <v>45.024999999999999</v>
+      </c>
+      <c r="AL68" s="7">
+        <f>AL56+1.86</f>
+        <v>8.379999999999999</v>
+      </c>
       <c r="AM68" s="41">
         <f t="shared" si="79"/>
-        <v>0</v>
-      </c>
-      <c r="AN68" s="7"/>
-      <c r="AO68" s="7"/>
-      <c r="AP68" s="7"/>
-      <c r="AQ68" s="7"/>
+        <v>1.0622002499999998E-2</v>
+      </c>
+      <c r="AN68" s="7">
+        <v>201.93</v>
+      </c>
+      <c r="AO68" s="7">
+        <v>69.75</v>
+      </c>
+      <c r="AP68" s="7">
+        <v>460</v>
+      </c>
+      <c r="AQ68" s="7">
+        <v>2025</v>
+      </c>
       <c r="AR68" s="41">
         <v>51.660000000000082</v>
       </c>
       <c r="AS68" s="41">
-        <f t="shared" si="82"/>
-        <v>-51.660000000000082</v>
+        <f>AQ68-AR68</f>
+        <v>1973.34</v>
       </c>
       <c r="AT68" s="41">
         <f t="shared" si="36"/>
-        <v>-187.96</v>
+        <v>13.969999999999999</v>
       </c>
       <c r="AU68" s="41">
         <f t="shared" si="37"/>
-        <v>-56.59</v>
+        <v>13.159999999999997</v>
       </c>
       <c r="AV68" s="41">
         <f t="shared" si="65"/>
-        <v>476</v>
+        <v>16</v>
       </c>
       <c r="AW68" s="26">
         <v>15</v>
@@ -16183,48 +16660,50 @@
       <c r="BB68" s="23">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BC68" s="12"/>
+      <c r="BC68" s="12">
+        <v>8.0999999999999996E-3</v>
+      </c>
       <c r="BD68" s="5"/>
       <c r="BE68" s="23"/>
       <c r="BF68" s="12">
+        <f t="shared" si="82"/>
+        <v>1.1160183959999999E-2</v>
+      </c>
+      <c r="BG68" s="13">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG68" s="13">
-        <f t="shared" si="84"/>
-        <v>0</v>
+        <v>16.070664902399997</v>
       </c>
       <c r="BH68" s="13">
         <f t="shared" si="41"/>
-        <v>1535</v>
-      </c>
-      <c r="BI68" s="14" t="str">
-        <f t="shared" ref="BI68:BI80" si="88">IF(ISBLANK(AN68),"",IFERROR(AN68/BH68,0))</f>
-        <v/>
-      </c>
-      <c r="BJ68" s="14" t="str">
-        <f t="shared" ref="BJ68:BJ80" si="89">IF(ISBLANK(AN68),"",AN68/AX68)</f>
-        <v/>
+        <v>1888.3559999999998</v>
+      </c>
+      <c r="BI68" s="14">
+        <f t="shared" ref="BI68:BI80" si="87">IF(ISBLANK(AN68),"",IFERROR(AN68/BH68,0))</f>
+        <v>0.10693428569612935</v>
+      </c>
+      <c r="BJ68" s="14">
+        <f t="shared" ref="BJ68:BJ80" si="88">IF(ISBLANK(AN68),"",AN68/AX68)</f>
+        <v>0.11878235294117648</v>
       </c>
       <c r="BK68" s="14">
-        <f t="shared" si="85"/>
-        <v>0</v>
+        <f t="shared" si="84"/>
+        <v>15.295683599999997</v>
       </c>
       <c r="BL68" s="14">
-        <f t="shared" ref="BL68:BL80" si="90">IF(B68="Python",BC68*BH68/24/60,"")</f>
-        <v>0</v>
+        <f t="shared" ref="BL68:BL80" si="89">IF(B68="Python",BC68*BH68/24/60,"")</f>
+        <v>1.0622002499999998E-2</v>
       </c>
       <c r="BM68" s="48" t="str">
         <f t="shared" si="31"/>
         <v/>
       </c>
       <c r="BN68" s="36" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO68" s="14">
         <f t="shared" si="47"/>
-        <v>11.512499999999999</v>
+        <v>11.046882599999998</v>
       </c>
       <c r="BP68" s="52" t="str">
         <f t="shared" si="28"/>
@@ -16232,15 +16711,15 @@
       </c>
       <c r="BQ68" s="29">
         <f t="shared" si="80"/>
-        <v>0</v>
+        <v>27.589616883116879</v>
       </c>
       <c r="BR68" s="38">
         <f t="shared" si="81"/>
-        <v>0</v>
+        <v>1.0622002499999998E-2</v>
       </c>
       <c r="BS68" s="31">
-        <f t="shared" si="87"/>
-        <v>11.512499999999999</v>
+        <f t="shared" si="86"/>
+        <v>11.046882599999998</v>
       </c>
     </row>
     <row r="69" spans="1:71" x14ac:dyDescent="0.3">
@@ -16257,70 +16736,137 @@
         <v>11</v>
       </c>
       <c r="E69" s="3"/>
-      <c r="F69" s="60"/>
+      <c r="F69" s="60">
+        <v>45544.577546296299</v>
+      </c>
       <c r="G69" s="63">
         <v>6057.48</v>
       </c>
       <c r="H69" s="6"/>
-      <c r="I69" s="6"/>
-      <c r="J69" s="6"/>
-      <c r="K69" s="6"/>
-      <c r="L69" s="6"/>
-      <c r="M69" s="6"/>
-      <c r="N69" s="6"/>
-      <c r="O69" s="6"/>
-      <c r="P69" s="6"/>
-      <c r="Q69" s="6"/>
+      <c r="I69" s="6">
+        <v>5674.0649999999996</v>
+      </c>
+      <c r="J69" s="6">
+        <v>22.2</v>
+      </c>
+      <c r="K69" s="6">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="L69" s="6">
+        <v>89.7</v>
+      </c>
+      <c r="M69" s="6">
+        <v>17</v>
+      </c>
+      <c r="N69" s="6">
+        <v>355</v>
+      </c>
+      <c r="O69" s="6">
+        <v>1.72</v>
+      </c>
+      <c r="P69" s="6">
+        <v>0.21</v>
+      </c>
+      <c r="Q69" s="6">
+        <v>0</v>
+      </c>
       <c r="R69" s="6"/>
-      <c r="S69" s="6"/>
-      <c r="T69" s="6"/>
-      <c r="U69" s="6"/>
-      <c r="V69" s="6"/>
-      <c r="W69" s="6"/>
-      <c r="X69" s="6"/>
-      <c r="Y69" s="6"/>
-      <c r="Z69" s="6"/>
-      <c r="AA69" s="6"/>
-      <c r="AB69" s="6"/>
-      <c r="AC69" s="6"/>
-      <c r="AD69" s="16"/>
-      <c r="AE69" s="6"/>
-      <c r="AF69" s="6"/>
-      <c r="AG69" s="6"/>
+      <c r="S69" s="6">
+        <v>0.17</v>
+      </c>
+      <c r="T69" s="6">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="U69" s="6">
+        <v>2.37</v>
+      </c>
+      <c r="V69" s="6">
+        <v>7.2590000000000003</v>
+      </c>
+      <c r="W69" s="6">
+        <v>51.3</v>
+      </c>
+      <c r="X69" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y69" s="6">
+        <v>3.44</v>
+      </c>
+      <c r="Z69" s="6">
+        <v>151.1</v>
+      </c>
+      <c r="AA69" s="6">
+        <v>22.4</v>
+      </c>
+      <c r="AB69" s="6">
+        <v>45</v>
+      </c>
+      <c r="AC69" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="16">
+        <v>7.3</v>
+      </c>
+      <c r="AE69" s="6">
+        <v>299</v>
+      </c>
+      <c r="AF69" s="6">
+        <v>40.5</v>
+      </c>
+      <c r="AG69" s="6">
+        <v>7.3</v>
+      </c>
       <c r="AH69" s="40">
         <f>AF69/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI69" s="6"/>
-      <c r="AJ69" s="6"/>
-      <c r="AK69" s="44"/>
-      <c r="AL69" s="6"/>
+        <v>0.40500000000000003</v>
+      </c>
+      <c r="AI69" s="6">
+        <v>34</v>
+      </c>
+      <c r="AJ69" s="6">
+        <v>27.91</v>
+      </c>
+      <c r="AK69" s="44">
+        <v>47.91</v>
+      </c>
+      <c r="AL69" s="6">
+        <f>AL51+3.09</f>
+        <v>8.379999999999999</v>
+      </c>
       <c r="AM69" s="42">
         <f>BR69</f>
-        <v>0</v>
-      </c>
-      <c r="AN69" s="6"/>
-      <c r="AO69" s="6"/>
-      <c r="AP69" s="6"/>
-      <c r="AQ69" s="6"/>
+        <v>2.7214024885993001E-2</v>
+      </c>
+      <c r="AN69" s="6">
+        <v>181.29</v>
+      </c>
+      <c r="AO69" s="6">
+        <v>73.31</v>
+      </c>
+      <c r="AP69" s="6">
+        <v>485</v>
+      </c>
+      <c r="AQ69" s="6">
+        <v>1912</v>
+      </c>
       <c r="AR69" s="40">
         <v>137.11999999999989</v>
       </c>
       <c r="AS69" s="40">
-        <f t="shared" si="82"/>
-        <v>-137.11999999999989</v>
+        <f t="shared" ref="AS69:AS80" si="90">AQ69-AR69</f>
+        <v>1774.88</v>
       </c>
       <c r="AT69" s="40">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>11.400000000000006</v>
       </c>
       <c r="AU69" s="40">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AV69" s="40">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AW69" s="24">
         <v>15</v>
@@ -16341,42 +16887,47 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC69" s="8"/>
-      <c r="BD69" s="9"/>
-      <c r="BE69" s="21"/>
+      <c r="BD69" s="46">
+        <f>BM69*24*60/BH69</f>
+        <v>2.1082524120846741E-2</v>
+      </c>
+      <c r="BE69" s="22">
+        <f>BP69/BH69</f>
+        <v>5.1774073553105659E-3</v>
+      </c>
       <c r="BF69" s="8">
+        <f t="shared" si="82"/>
+        <v>1.1097035999999998E-2</v>
+      </c>
+      <c r="BG69" s="9">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG69" s="9">
-        <f t="shared" si="84"/>
-        <v>0</v>
+        <v>15.979731839999996</v>
       </c>
       <c r="BH69" s="9">
         <f t="shared" si="41"/>
-        <v>1520</v>
-      </c>
-      <c r="BI69" s="10" t="str">
+        <v>1858.8</v>
+      </c>
+      <c r="BI69" s="10">
+        <f t="shared" si="87"/>
+        <v>9.7530664945125883E-2</v>
+      </c>
+      <c r="BJ69" s="10">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ69" s="10" t="str">
+        <v>0.10664117647058823</v>
+      </c>
+      <c r="BK69" s="10">
+        <f t="shared" si="84"/>
+        <v>39.188195835829923</v>
+      </c>
+      <c r="BL69" s="10" t="str">
         <f t="shared" si="89"/>
         <v/>
       </c>
-      <c r="BK69" s="10">
+      <c r="BM69" s="10">
+        <v>2.7214024885993001E-2</v>
+      </c>
+      <c r="BN69" s="35" t="str">
         <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL69" s="10" t="str">
-        <f t="shared" si="90"/>
-        <v/>
-      </c>
-      <c r="BM69" s="10">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="BN69" s="35" t="str">
-        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="BO69" s="10" t="str">
@@ -16384,20 +16935,19 @@
         <v/>
       </c>
       <c r="BP69" s="50">
-        <f t="shared" si="28"/>
-        <v>0</v>
+        <v>9.6237647920512792</v>
       </c>
       <c r="BQ69" s="27">
         <f>IF(BL69&lt;&gt;"",BL69/0.000385,IF(BM69&lt;&gt;"",BM69/0.000385,BN69/0.000385))</f>
-        <v>0</v>
+        <v>70.685778924657143</v>
       </c>
       <c r="BR69" s="37">
         <f>IF(BL69&lt;&gt;"",BL69,IF(BM69&lt;&gt;"",BM69,BN69))</f>
-        <v>0</v>
+        <v>2.7214024885993001E-2</v>
       </c>
       <c r="BS69" s="32">
-        <f t="shared" si="87"/>
-        <v>0</v>
+        <f t="shared" si="86"/>
+        <v>9.6237647920512792</v>
       </c>
     </row>
     <row r="70" spans="1:71" x14ac:dyDescent="0.3">
@@ -16413,70 +16963,137 @@
       <c r="D70">
         <v>11</v>
       </c>
-      <c r="F70" s="61"/>
+      <c r="F70" s="61">
+        <v>45544.6039467593</v>
+      </c>
       <c r="G70" s="64">
         <v>6057.48</v>
       </c>
       <c r="H70" s="44"/>
-      <c r="I70" s="44"/>
-      <c r="J70" s="44"/>
-      <c r="K70" s="44"/>
-      <c r="L70" s="44"/>
-      <c r="M70" s="44"/>
-      <c r="N70" s="44"/>
-      <c r="O70" s="44"/>
-      <c r="P70" s="44"/>
-      <c r="Q70" s="44"/>
+      <c r="I70" s="44">
+        <v>6019.3950000000004</v>
+      </c>
+      <c r="J70" s="44">
+        <v>18.8</v>
+      </c>
+      <c r="K70" s="44">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="L70" s="44">
+        <v>90.8</v>
+      </c>
+      <c r="M70" s="44">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="N70" s="44">
+        <v>351</v>
+      </c>
+      <c r="O70" s="44">
+        <v>2.5</v>
+      </c>
+      <c r="P70" s="44">
+        <v>0.21</v>
+      </c>
+      <c r="Q70" s="44">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="R70" s="44"/>
-      <c r="S70" s="44"/>
-      <c r="T70" s="44"/>
-      <c r="U70" s="44"/>
-      <c r="V70" s="44"/>
-      <c r="W70" s="44"/>
-      <c r="X70" s="44"/>
-      <c r="Y70" s="44"/>
-      <c r="Z70" s="44"/>
-      <c r="AA70" s="44"/>
-      <c r="AB70" s="44"/>
-      <c r="AC70" s="44"/>
-      <c r="AD70" s="17"/>
-      <c r="AE70" s="44"/>
-      <c r="AF70" s="44"/>
-      <c r="AG70" s="44"/>
+      <c r="S70" s="44">
+        <v>0</v>
+      </c>
+      <c r="T70" s="44">
+        <v>0.16</v>
+      </c>
+      <c r="U70" s="44">
+        <v>0</v>
+      </c>
+      <c r="V70" s="44">
+        <v>7.2969999999999997</v>
+      </c>
+      <c r="W70" s="44">
+        <v>113.3</v>
+      </c>
+      <c r="X70" s="44">
+        <v>68.3</v>
+      </c>
+      <c r="Y70" s="44">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="Z70" s="44">
+        <v>155.69999999999999</v>
+      </c>
+      <c r="AA70" s="44">
+        <v>54</v>
+      </c>
+      <c r="AB70" s="44">
+        <v>99.3</v>
+      </c>
+      <c r="AC70" s="44">
+        <v>55.7</v>
+      </c>
+      <c r="AD70" s="17">
+        <v>7.34</v>
+      </c>
+      <c r="AE70" s="44">
+        <v>300</v>
+      </c>
+      <c r="AF70" s="44">
+        <v>48.3</v>
+      </c>
+      <c r="AG70" s="44">
+        <v>7.27</v>
+      </c>
       <c r="AH70" s="45">
         <f t="shared" ref="AH70:AH74" si="91">AF70/100</f>
-        <v>0</v>
-      </c>
-      <c r="AI70" s="44"/>
-      <c r="AJ70" s="44"/>
-      <c r="AK70" s="44"/>
-      <c r="AL70" s="44"/>
+        <v>0.48299999999999998</v>
+      </c>
+      <c r="AI70" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ70" s="44">
+        <v>24.57</v>
+      </c>
+      <c r="AK70" s="44">
+        <v>27.96</v>
+      </c>
+      <c r="AL70" s="44">
+        <f>AL52+3.01</f>
+        <v>6.01</v>
+      </c>
       <c r="AM70" s="45">
         <f t="shared" ref="AM70:AM74" si="92">BR70</f>
-        <v>0</v>
-      </c>
-      <c r="AN70" s="44"/>
-      <c r="AO70" s="44"/>
-      <c r="AP70" s="44"/>
-      <c r="AQ70" s="44"/>
+        <v>1.7809574480595398E-2</v>
+      </c>
+      <c r="AN70" s="44">
+        <v>205.53</v>
+      </c>
+      <c r="AO70" s="44">
+        <v>79.069999999999993</v>
+      </c>
+      <c r="AP70" s="44">
+        <v>458</v>
+      </c>
+      <c r="AQ70" s="44">
+        <v>1845</v>
+      </c>
       <c r="AR70" s="45">
         <v>45.769999999999982</v>
       </c>
       <c r="AS70" s="45">
-        <f t="shared" si="82"/>
-        <v>-45.769999999999982</v>
+        <f t="shared" si="90"/>
+        <v>1799.23</v>
       </c>
       <c r="AT70" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>20.22</v>
       </c>
       <c r="AU70" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>10.819999999999993</v>
       </c>
       <c r="AV70" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="AW70" s="25">
         <v>15</v>
@@ -16497,42 +17114,47 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC70" s="11"/>
-      <c r="BD70" s="46"/>
-      <c r="BE70" s="22"/>
+      <c r="BD70" s="46">
+        <f>BM70*24*60/BH70</f>
+        <v>1.3764820277626683E-2</v>
+      </c>
+      <c r="BE70" s="22">
+        <f>BP70/BH70</f>
+        <v>4.396909262276265E-3</v>
+      </c>
       <c r="BF70" s="11">
+        <f t="shared" si="82"/>
+        <v>9.5579081999999996E-3</v>
+      </c>
+      <c r="BG70" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG70" s="46">
-        <f t="shared" si="84"/>
-        <v>0</v>
+        <v>13.763387807999999</v>
       </c>
       <c r="BH70" s="46">
         <f t="shared" si="41"/>
-        <v>1520</v>
-      </c>
-      <c r="BI70" s="47" t="str">
+        <v>1863.1399999999999</v>
+      </c>
+      <c r="BI70" s="47">
+        <f t="shared" si="87"/>
+        <v>0.1103137713752053</v>
+      </c>
+      <c r="BJ70" s="47">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ70" s="47" t="str">
+        <v>0.12090000000000001</v>
+      </c>
+      <c r="BK70" s="47">
+        <f t="shared" si="84"/>
+        <v>25.645787252057374</v>
+      </c>
+      <c r="BL70" s="47" t="str">
         <f t="shared" si="89"/>
         <v/>
       </c>
-      <c r="BK70" s="47">
+      <c r="BM70" s="47">
+        <v>1.7809574480595398E-2</v>
+      </c>
+      <c r="BN70" s="48" t="str">
         <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL70" s="47" t="str">
-        <f t="shared" si="90"/>
-        <v/>
-      </c>
-      <c r="BM70" s="47">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="BN70" s="48" t="str">
-        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="BO70" s="47" t="str">
@@ -16540,20 +17162,19 @@
         <v/>
       </c>
       <c r="BP70" s="51">
-        <f t="shared" ref="BP70:BP80" si="93">IF(B70="Julia",BE70*BH70,"")</f>
-        <v>0</v>
+        <v>8.1920575229174002</v>
       </c>
       <c r="BQ70" s="28">
-        <f t="shared" ref="BQ70:BQ74" si="94">IF(BL70&lt;&gt;"",BL70/0.000385,IF(BM70&lt;&gt;"",BM70/0.000385,BN70/0.000385))</f>
-        <v>0</v>
+        <f t="shared" ref="BQ70:BQ74" si="93">IF(BL70&lt;&gt;"",BL70/0.000385,IF(BM70&lt;&gt;"",BM70/0.000385,BN70/0.000385))</f>
+        <v>46.258635014533503</v>
       </c>
       <c r="BR70" s="49">
-        <f t="shared" ref="BR70:BR74" si="95">IF(BL70&lt;&gt;"",BL70,IF(BM70&lt;&gt;"",BM70,BN70))</f>
-        <v>0</v>
+        <f t="shared" ref="BR70:BR74" si="94">IF(BL70&lt;&gt;"",BL70,IF(BM70&lt;&gt;"",BM70,BN70))</f>
+        <v>1.7809574480595398E-2</v>
       </c>
       <c r="BS70" s="30">
-        <f t="shared" si="87"/>
-        <v>0</v>
+        <f t="shared" si="86"/>
+        <v>8.1920575229174002</v>
       </c>
     </row>
     <row r="71" spans="1:71" x14ac:dyDescent="0.3">
@@ -16569,70 +17190,137 @@
       <c r="D71">
         <v>11</v>
       </c>
-      <c r="F71" s="61"/>
+      <c r="F71" s="61">
+        <v>45544.5913657407</v>
+      </c>
       <c r="G71" s="64">
         <v>6057.48</v>
       </c>
       <c r="H71" s="44"/>
-      <c r="I71" s="44"/>
-      <c r="J71" s="44"/>
-      <c r="K71" s="44"/>
-      <c r="L71" s="44"/>
-      <c r="M71" s="44"/>
-      <c r="N71" s="44"/>
-      <c r="O71" s="44"/>
-      <c r="P71" s="44"/>
-      <c r="Q71" s="44"/>
+      <c r="I71" s="44">
+        <v>5282.2049999999999</v>
+      </c>
+      <c r="J71" s="44">
+        <v>19.2</v>
+      </c>
+      <c r="K71" s="44">
+        <v>16.5</v>
+      </c>
+      <c r="L71" s="44">
+        <v>86</v>
+      </c>
+      <c r="M71" s="44">
+        <v>19</v>
+      </c>
+      <c r="N71" s="44">
+        <v>446</v>
+      </c>
+      <c r="O71" s="44">
+        <v>2.98</v>
+      </c>
+      <c r="P71" s="44">
+        <v>0.2</v>
+      </c>
+      <c r="Q71" s="44">
+        <v>2.21</v>
+      </c>
       <c r="R71" s="44"/>
-      <c r="S71" s="44"/>
-      <c r="T71" s="44"/>
-      <c r="U71" s="44"/>
-      <c r="V71" s="44"/>
-      <c r="W71" s="44"/>
-      <c r="X71" s="44"/>
-      <c r="Y71" s="44"/>
-      <c r="Z71" s="44"/>
-      <c r="AA71" s="44"/>
-      <c r="AB71" s="44"/>
-      <c r="AC71" s="44"/>
-      <c r="AD71" s="17"/>
-      <c r="AE71" s="44"/>
-      <c r="AF71" s="44"/>
-      <c r="AG71" s="44"/>
+      <c r="S71" s="44">
+        <v>1</v>
+      </c>
+      <c r="T71" s="44">
+        <v>3.23</v>
+      </c>
+      <c r="U71" s="44">
+        <v>1.39</v>
+      </c>
+      <c r="V71" s="44">
+        <v>7.266</v>
+      </c>
+      <c r="W71" s="44">
+        <v>127.3</v>
+      </c>
+      <c r="X71" s="44">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="Y71" s="44">
+        <v>1.48</v>
+      </c>
+      <c r="Z71" s="44">
+        <v>178.2</v>
+      </c>
+      <c r="AA71" s="44">
+        <v>56.4</v>
+      </c>
+      <c r="AB71" s="44">
+        <v>111.7</v>
+      </c>
+      <c r="AC71" s="44">
+        <v>16.3</v>
+      </c>
+      <c r="AD71" s="17">
+        <v>7.3070000000000004</v>
+      </c>
+      <c r="AE71" s="44">
+        <v>298</v>
+      </c>
+      <c r="AF71" s="44">
+        <v>50</v>
+      </c>
+      <c r="AG71" s="44">
+        <v>7.27</v>
+      </c>
       <c r="AH71" s="45">
         <f t="shared" si="91"/>
-        <v>0</v>
-      </c>
-      <c r="AI71" s="44"/>
-      <c r="AJ71" s="44"/>
-      <c r="AK71" s="44"/>
-      <c r="AL71" s="44"/>
+        <v>0.5</v>
+      </c>
+      <c r="AI71" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ71" s="44">
+        <v>38.049999999999997</v>
+      </c>
+      <c r="AK71" s="44">
+        <v>5.17</v>
+      </c>
+      <c r="AL71" s="44">
+        <f>AL53+3.04</f>
+        <v>9.6999999999999993</v>
+      </c>
       <c r="AM71" s="45">
         <f t="shared" si="92"/>
-        <v>0</v>
-      </c>
-      <c r="AN71" s="44"/>
-      <c r="AO71" s="44"/>
-      <c r="AP71" s="44"/>
-      <c r="AQ71" s="44"/>
+        <v>3.24883333333333E-2</v>
+      </c>
+      <c r="AN71" s="44">
+        <v>287.8</v>
+      </c>
+      <c r="AO71" s="44">
+        <v>88.58</v>
+      </c>
+      <c r="AP71" s="44">
+        <v>338</v>
+      </c>
+      <c r="AQ71" s="44">
+        <v>1970</v>
+      </c>
       <c r="AR71" s="45">
         <v>84.700000000000045</v>
       </c>
       <c r="AS71" s="45">
-        <f t="shared" si="82"/>
-        <v>-84.700000000000045</v>
+        <f t="shared" si="90"/>
+        <v>1885.3</v>
       </c>
       <c r="AT71" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>38.360000000000014</v>
       </c>
       <c r="AU71" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>3.8199999999999932</v>
       </c>
       <c r="AV71" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="AW71" s="25">
         <v>15</v>
@@ -16653,42 +17341,47 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BC71" s="11"/>
-      <c r="BD71" s="46"/>
-      <c r="BE71" s="22"/>
+      <c r="BD71" s="46">
+        <f>BM71*24*60/BH71</f>
+        <v>2.3999999999999973E-2</v>
+      </c>
+      <c r="BE71" s="22">
+        <f>BP71/BH71</f>
+        <v>5.1005554585699941E-3</v>
+      </c>
       <c r="BF71" s="11">
+        <f t="shared" si="82"/>
+        <v>9.6490350000000003E-3</v>
+      </c>
+      <c r="BG71" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG71" s="46">
-        <f t="shared" si="84"/>
-        <v>0</v>
+        <v>13.894610400000001</v>
       </c>
       <c r="BH71" s="46">
         <f t="shared" si="41"/>
-        <v>1520</v>
-      </c>
-      <c r="BI71" s="47" t="str">
+        <v>1949.3000000000002</v>
+      </c>
+      <c r="BI71" s="47">
+        <f t="shared" si="87"/>
+        <v>0.14764274354896628</v>
+      </c>
+      <c r="BJ71" s="47">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ71" s="47" t="str">
+        <v>0.16929411764705882</v>
+      </c>
+      <c r="BK71" s="47">
+        <f t="shared" si="84"/>
+        <v>46.783199999999951</v>
+      </c>
+      <c r="BL71" s="47" t="str">
         <f t="shared" si="89"/>
         <v/>
       </c>
-      <c r="BK71" s="47">
+      <c r="BM71" s="47">
+        <v>3.24883333333333E-2</v>
+      </c>
+      <c r="BN71" s="48" t="str">
         <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL71" s="47" t="str">
-        <f t="shared" si="90"/>
-        <v/>
-      </c>
-      <c r="BM71" s="47">
-        <f t="shared" ref="BM71:BM80" si="96">IF(B71="Julia",BD71*BH71/24/60,"")</f>
-        <v>0</v>
-      </c>
-      <c r="BN71" s="48" t="str">
-        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="BO71" s="47" t="str">
@@ -16696,20 +17389,19 @@
         <v/>
       </c>
       <c r="BP71" s="51">
+        <v>9.9425127553904904</v>
+      </c>
+      <c r="BQ71" s="28">
         <f t="shared" si="93"/>
-        <v>0</v>
-      </c>
-      <c r="BQ71" s="28">
+        <v>84.385281385281303</v>
+      </c>
+      <c r="BR71" s="49">
         <f t="shared" si="94"/>
-        <v>0</v>
-      </c>
-      <c r="BR71" s="49">
-        <f t="shared" si="95"/>
-        <v>0</v>
+        <v>3.24883333333333E-2</v>
       </c>
       <c r="BS71" s="30">
-        <f t="shared" si="87"/>
-        <v>0</v>
+        <f t="shared" si="86"/>
+        <v>9.9425127553904904</v>
       </c>
     </row>
     <row r="72" spans="1:71" x14ac:dyDescent="0.3">
@@ -16725,70 +17417,137 @@
       <c r="D72">
         <v>11</v>
       </c>
-      <c r="F72" s="61"/>
+      <c r="F72" s="61">
+        <v>45544.610312500001</v>
+      </c>
       <c r="G72" s="64">
         <v>6057.48</v>
       </c>
       <c r="H72" s="44"/>
-      <c r="I72" s="44"/>
-      <c r="J72" s="44"/>
-      <c r="K72" s="44"/>
-      <c r="L72" s="44"/>
-      <c r="M72" s="44"/>
-      <c r="N72" s="44"/>
-      <c r="O72" s="44"/>
-      <c r="P72" s="44"/>
-      <c r="Q72" s="44"/>
+      <c r="I72" s="44">
+        <v>5403.24</v>
+      </c>
+      <c r="J72" s="44">
+        <v>19.5</v>
+      </c>
+      <c r="K72" s="44">
+        <v>17.2</v>
+      </c>
+      <c r="L72" s="44">
+        <v>88</v>
+      </c>
+      <c r="M72" s="44">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="N72" s="44">
+        <v>437</v>
+      </c>
+      <c r="O72" s="44">
+        <v>2.12</v>
+      </c>
+      <c r="P72" s="44">
+        <v>0.2</v>
+      </c>
+      <c r="Q72" s="44">
+        <v>0.77</v>
+      </c>
       <c r="R72" s="44"/>
-      <c r="S72" s="44"/>
-      <c r="T72" s="44"/>
-      <c r="U72" s="44"/>
-      <c r="V72" s="44"/>
-      <c r="W72" s="44"/>
-      <c r="X72" s="44"/>
-      <c r="Y72" s="44"/>
-      <c r="Z72" s="44"/>
-      <c r="AA72" s="44"/>
-      <c r="AB72" s="44"/>
-      <c r="AC72" s="44"/>
-      <c r="AD72" s="17"/>
-      <c r="AE72" s="44"/>
-      <c r="AF72" s="44"/>
-      <c r="AG72" s="44"/>
+      <c r="S72" s="44">
+        <v>0.83</v>
+      </c>
+      <c r="T72" s="44">
+        <v>2.97</v>
+      </c>
+      <c r="U72" s="44">
+        <v>2.21</v>
+      </c>
+      <c r="V72" s="44">
+        <v>7.2830000000000004</v>
+      </c>
+      <c r="W72" s="44">
+        <v>125.9</v>
+      </c>
+      <c r="X72" s="44">
+        <v>102.1</v>
+      </c>
+      <c r="Y72" s="44">
+        <v>1.45</v>
+      </c>
+      <c r="Z72" s="44">
+        <v>182.7</v>
+      </c>
+      <c r="AA72" s="44">
+        <v>58</v>
+      </c>
+      <c r="AB72" s="44">
+        <v>110.4</v>
+      </c>
+      <c r="AC72" s="44">
+        <v>85.6</v>
+      </c>
+      <c r="AD72" s="17">
+        <v>7.3239999999999998</v>
+      </c>
+      <c r="AE72" s="44">
+        <v>302</v>
+      </c>
+      <c r="AF72" s="44">
+        <v>100</v>
+      </c>
+      <c r="AG72" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH72" s="45">
         <f t="shared" si="91"/>
-        <v>0</v>
-      </c>
-      <c r="AI72" s="44"/>
-      <c r="AJ72" s="44"/>
-      <c r="AK72" s="44"/>
-      <c r="AL72" s="44"/>
+        <v>1</v>
+      </c>
+      <c r="AI72" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ72" s="44">
+        <v>43.09</v>
+      </c>
+      <c r="AK72" s="44">
+        <v>17.54</v>
+      </c>
+      <c r="AL72" s="44">
+        <f>AL54+3.1</f>
+        <v>9.86</v>
+      </c>
       <c r="AM72" s="45">
         <f t="shared" si="92"/>
         <v>0</v>
       </c>
-      <c r="AN72" s="44"/>
-      <c r="AO72" s="44"/>
-      <c r="AP72" s="44"/>
-      <c r="AQ72" s="44"/>
+      <c r="AN72" s="44">
+        <v>273.05</v>
+      </c>
+      <c r="AO72" s="44">
+        <v>79.709999999999994</v>
+      </c>
+      <c r="AP72" s="44">
+        <v>362</v>
+      </c>
+      <c r="AQ72" s="44">
+        <v>1953</v>
+      </c>
       <c r="AR72" s="45">
         <v>47.420000000000073</v>
       </c>
       <c r="AS72" s="45">
-        <f t="shared" si="82"/>
-        <v>-47.420000000000073</v>
+        <f t="shared" si="90"/>
+        <v>1905.58</v>
       </c>
       <c r="AT72" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>39.120000000000005</v>
       </c>
       <c r="AU72" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>8.8399999999999892</v>
       </c>
       <c r="AV72" s="45">
         <f t="shared" si="65"/>
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="AW72" s="25">
         <v>15</v>
@@ -16811,60 +17570,60 @@
       <c r="BC72" s="11"/>
       <c r="BE72" s="22"/>
       <c r="BF72" s="11">
+        <f t="shared" si="82"/>
+        <v>1.002717E-2</v>
+      </c>
+      <c r="BG72" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG72" s="46">
+        <v>14.4391248</v>
+      </c>
+      <c r="BH72" s="46">
+        <f t="shared" ref="BH72:BH80" si="95">AX72+SUM(AJ72:AL72,AN72:AO72)-(AW72*(D72+1))</f>
+        <v>1943.25</v>
+      </c>
+      <c r="BI72" s="47">
+        <f t="shared" si="87"/>
+        <v>0.14051202881770231</v>
+      </c>
+      <c r="BJ72" s="47">
+        <f t="shared" si="88"/>
+        <v>0.16061764705882353</v>
+      </c>
+      <c r="BK72" s="47">
         <f t="shared" si="84"/>
         <v>0</v>
       </c>
-      <c r="BH72" s="46">
-        <f t="shared" ref="BH72:BH80" si="97">AX72+SUM(AJ72:AL72,AN72:AO72)-(AW72*(D72+1))</f>
-        <v>1520</v>
-      </c>
-      <c r="BI72" s="47" t="str">
-        <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ72" s="47" t="str">
+      <c r="BL72" s="47">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK72" s="47">
+        <v>0</v>
+      </c>
+      <c r="BM72" s="48" t="str">
+        <f t="shared" ref="BM71:BM80" si="96">IF(B72="Julia",BD72*BH72/24/60,"")</f>
+        <v/>
+      </c>
+      <c r="BN72" s="48" t="str">
         <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL72" s="47">
-        <f t="shared" si="90"/>
-        <v>0</v>
-      </c>
-      <c r="BM72" s="48" t="str">
-        <f t="shared" si="96"/>
-        <v/>
-      </c>
-      <c r="BN72" s="48" t="str">
-        <f t="shared" si="86"/>
         <v/>
       </c>
       <c r="BO72" s="47">
         <f t="shared" si="47"/>
-        <v>11.4</v>
+        <v>10.833618750000001</v>
       </c>
       <c r="BP72" s="51" t="str">
+        <f t="shared" ref="BP70:BP80" si="97">IF(B72="Julia",BE72*BH72,"")</f>
+        <v/>
+      </c>
+      <c r="BQ72" s="28">
         <f t="shared" si="93"/>
-        <v/>
-      </c>
-      <c r="BQ72" s="28">
+        <v>0</v>
+      </c>
+      <c r="BR72" s="49">
         <f t="shared" si="94"/>
         <v>0</v>
       </c>
-      <c r="BR72" s="49">
-        <f t="shared" si="95"/>
-        <v>0</v>
-      </c>
       <c r="BS72" s="30">
-        <f t="shared" si="87"/>
-        <v>11.4</v>
+        <f t="shared" si="86"/>
+        <v>10.833618750000001</v>
       </c>
     </row>
     <row r="73" spans="1:71" x14ac:dyDescent="0.3">
@@ -16880,70 +17639,133 @@
       <c r="D73">
         <v>11</v>
       </c>
-      <c r="F73" s="61"/>
+      <c r="F73" s="61">
+        <v>45544.616192129601</v>
+      </c>
       <c r="G73" s="64">
         <v>6057.48</v>
       </c>
       <c r="H73" s="44"/>
-      <c r="I73" s="44"/>
-      <c r="J73" s="44"/>
-      <c r="K73" s="44"/>
-      <c r="L73" s="44"/>
-      <c r="M73" s="44"/>
-      <c r="N73" s="44"/>
+      <c r="I73" s="44">
+        <v>2556.4050000000002</v>
+      </c>
+      <c r="J73" s="44">
+        <v>20.2</v>
+      </c>
+      <c r="K73" s="44">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="L73" s="44">
+        <v>2.71</v>
+      </c>
+      <c r="M73" s="44">
+        <v>13.7</v>
+      </c>
+      <c r="N73" s="44">
+        <v>869</v>
+      </c>
       <c r="O73" s="44"/>
-      <c r="P73" s="44"/>
-      <c r="Q73" s="44"/>
+      <c r="P73" s="44">
+        <v>0.23</v>
+      </c>
+      <c r="Q73" s="44">
+        <v>6.87</v>
+      </c>
       <c r="R73" s="44"/>
-      <c r="S73" s="44"/>
-      <c r="T73" s="44"/>
+      <c r="S73" s="44">
+        <v>0.97</v>
+      </c>
+      <c r="T73" s="44">
+        <v>4.58</v>
+      </c>
       <c r="U73" s="44"/>
-      <c r="V73" s="44"/>
-      <c r="W73" s="44"/>
-      <c r="X73" s="44"/>
-      <c r="Y73" s="44"/>
-      <c r="Z73" s="44"/>
-      <c r="AA73" s="44"/>
-      <c r="AB73" s="44"/>
-      <c r="AC73" s="44"/>
-      <c r="AD73" s="17"/>
-      <c r="AE73" s="44"/>
-      <c r="AF73" s="44"/>
-      <c r="AG73" s="44"/>
+      <c r="V73" s="44">
+        <v>7.2770000000000001</v>
+      </c>
+      <c r="W73" s="44">
+        <v>5.8</v>
+      </c>
+      <c r="X73" s="44">
+        <v>95.2</v>
+      </c>
+      <c r="Y73" s="44">
+        <v>7.36</v>
+      </c>
+      <c r="Z73" s="44">
+        <v>318.8</v>
+      </c>
+      <c r="AA73" s="44">
+        <v>2.6</v>
+      </c>
+      <c r="AB73" s="44">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="AC73" s="44">
+        <v>79.2</v>
+      </c>
+      <c r="AD73" s="17">
+        <v>7.3179999999999996</v>
+      </c>
+      <c r="AE73" s="44">
+        <v>299</v>
+      </c>
+      <c r="AF73" s="44">
+        <v>52.4</v>
+      </c>
+      <c r="AG73" s="44">
+        <v>7.3</v>
+      </c>
       <c r="AH73" s="45">
         <f t="shared" si="91"/>
-        <v>0</v>
-      </c>
-      <c r="AI73" s="44"/>
-      <c r="AJ73" s="44"/>
-      <c r="AK73" s="44"/>
-      <c r="AL73" s="44"/>
+        <v>0.52400000000000002</v>
+      </c>
+      <c r="AI73" s="44">
+        <v>34</v>
+      </c>
+      <c r="AJ73" s="44">
+        <v>150</v>
+      </c>
+      <c r="AK73" s="44">
+        <v>9.64</v>
+      </c>
+      <c r="AL73" s="44">
+        <f>AL55+2.98</f>
+        <v>9.42</v>
+      </c>
       <c r="AM73" s="45">
         <f t="shared" si="92"/>
         <v>0</v>
       </c>
-      <c r="AN73" s="44"/>
-      <c r="AO73" s="44"/>
-      <c r="AP73" s="44"/>
-      <c r="AQ73" s="44"/>
+      <c r="AN73" s="44">
+        <v>310.07</v>
+      </c>
+      <c r="AO73" s="44">
+        <v>94.46</v>
+      </c>
+      <c r="AP73" s="44">
+        <v>295</v>
+      </c>
+      <c r="AQ73" s="44">
+        <v>2159</v>
+      </c>
       <c r="AR73" s="45">
         <v>133.55999999999995</v>
       </c>
       <c r="AS73" s="45">
-        <f t="shared" si="82"/>
-        <v>-133.55999999999995</v>
+        <f t="shared" si="90"/>
+        <v>2025.44</v>
       </c>
       <c r="AT73" s="45">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>48.389999999999986</v>
       </c>
       <c r="AU73" s="45">
         <f t="shared" si="37"/>
-        <v>0</v>
+        <v>16.64</v>
       </c>
       <c r="AV73" s="45">
         <f t="shared" ref="AV73:AV80" si="98">AP67-AP73</f>
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AW73" s="25">
         <v>15</v>
@@ -16966,31 +17788,31 @@
       <c r="BC73" s="11"/>
       <c r="BE73" s="22"/>
       <c r="BF73" s="11">
+        <f t="shared" si="82"/>
+        <v>3.4355811900000006E-4</v>
+      </c>
+      <c r="BG73" s="46">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG73" s="46">
+        <v>0.49472369136000011</v>
+      </c>
+      <c r="BH73" s="46">
+        <f t="shared" si="95"/>
+        <v>2093.59</v>
+      </c>
+      <c r="BI73" s="47">
+        <f t="shared" si="87"/>
+        <v>0.14810445216112036</v>
+      </c>
+      <c r="BJ73" s="47">
+        <f t="shared" si="88"/>
+        <v>0.18239411764705882</v>
+      </c>
+      <c r="BK73" s="47">
         <f t="shared" si="84"/>
         <v>0</v>
       </c>
-      <c r="BH73" s="46">
-        <f t="shared" si="97"/>
-        <v>1520</v>
-      </c>
-      <c r="BI73" s="47" t="str">
-        <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ73" s="47" t="str">
+      <c r="BL73" s="47">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK73" s="47">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL73" s="47">
-        <f t="shared" si="90"/>
         <v>0</v>
       </c>
       <c r="BM73" s="48" t="str">
@@ -16998,28 +17820,28 @@
         <v/>
       </c>
       <c r="BN73" s="48" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO73" s="47">
         <f t="shared" si="47"/>
-        <v>11.4</v>
+        <v>0</v>
       </c>
       <c r="BP73" s="51" t="str">
+        <f t="shared" si="97"/>
+        <v/>
+      </c>
+      <c r="BQ73" s="28">
         <f t="shared" si="93"/>
-        <v/>
-      </c>
-      <c r="BQ73" s="28">
+        <v>0</v>
+      </c>
+      <c r="BR73" s="49">
         <f t="shared" si="94"/>
         <v>0</v>
       </c>
-      <c r="BR73" s="49">
-        <f t="shared" si="95"/>
-        <v>0</v>
-      </c>
       <c r="BS73" s="30">
-        <f t="shared" si="87"/>
-        <v>11.4</v>
+        <f t="shared" si="86"/>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:71" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -17036,70 +17858,137 @@
         <v>11</v>
       </c>
       <c r="E74" s="5"/>
-      <c r="F74" s="62"/>
+      <c r="F74" s="62">
+        <v>45544.621018518519</v>
+      </c>
       <c r="G74" s="65">
         <v>6057.48</v>
       </c>
       <c r="H74" s="7"/>
-      <c r="I74" s="7"/>
-      <c r="J74" s="7"/>
-      <c r="K74" s="7"/>
-      <c r="L74" s="7"/>
-      <c r="M74" s="7"/>
-      <c r="N74" s="7"/>
-      <c r="O74" s="7"/>
-      <c r="P74" s="7"/>
-      <c r="Q74" s="7"/>
+      <c r="I74" s="7">
+        <v>6130.83</v>
+      </c>
+      <c r="J74" s="7">
+        <v>19.8</v>
+      </c>
+      <c r="K74" s="7">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="L74" s="7">
+        <v>90.2</v>
+      </c>
+      <c r="M74" s="7">
+        <v>17.8</v>
+      </c>
+      <c r="N74" s="7">
+        <v>359</v>
+      </c>
+      <c r="O74" s="7">
+        <v>1.91</v>
+      </c>
+      <c r="P74" s="7">
+        <v>0.18</v>
+      </c>
+      <c r="Q74" s="7">
+        <v>0.4</v>
+      </c>
       <c r="R74" s="7"/>
-      <c r="S74" s="7"/>
-      <c r="T74" s="7"/>
-      <c r="U74" s="7"/>
-      <c r="V74" s="7"/>
-      <c r="W74" s="7"/>
-      <c r="X74" s="7"/>
-      <c r="Y74" s="7"/>
-      <c r="Z74" s="7"/>
-      <c r="AA74" s="7"/>
-      <c r="AB74" s="7"/>
-      <c r="AC74" s="7"/>
-      <c r="AD74" s="18"/>
-      <c r="AE74" s="7"/>
-      <c r="AF74" s="7"/>
-      <c r="AG74" s="7"/>
+      <c r="S74" s="7">
+        <v>0.09</v>
+      </c>
+      <c r="T74" s="7">
+        <v>0.13</v>
+      </c>
+      <c r="U74" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="V74" s="7">
+        <v>7.2969999999999997</v>
+      </c>
+      <c r="W74" s="7">
+        <v>117.9</v>
+      </c>
+      <c r="X74" s="7">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="Y74" s="7">
+        <v>1.92</v>
+      </c>
+      <c r="Z74" s="7">
+        <v>159.1</v>
+      </c>
+      <c r="AA74" s="7">
+        <v>56.2</v>
+      </c>
+      <c r="AB74" s="7">
+        <v>103.4</v>
+      </c>
+      <c r="AC74" s="7">
+        <v>32.9</v>
+      </c>
+      <c r="AD74" s="18">
+        <v>7.3390000000000004</v>
+      </c>
+      <c r="AE74" s="7">
+        <v>298</v>
+      </c>
+      <c r="AF74" s="7">
+        <v>49.9</v>
+      </c>
+      <c r="AG74" s="7">
+        <v>7.29</v>
+      </c>
       <c r="AH74" s="41">
         <f t="shared" si="91"/>
-        <v>0</v>
-      </c>
-      <c r="AI74" s="7"/>
-      <c r="AJ74" s="7"/>
-      <c r="AK74" s="7"/>
-      <c r="AL74" s="7"/>
+        <v>0.499</v>
+      </c>
+      <c r="AI74" s="7">
+        <v>34</v>
+      </c>
+      <c r="AJ74" s="7">
+        <v>28.27</v>
+      </c>
+      <c r="AK74" s="7">
+        <v>45.05</v>
+      </c>
+      <c r="AL74" s="7">
+        <f>AL56+3.03</f>
+        <v>9.5499999999999989</v>
+      </c>
       <c r="AM74" s="41">
         <f t="shared" si="92"/>
         <v>0</v>
       </c>
-      <c r="AN74" s="7"/>
-      <c r="AO74" s="7"/>
-      <c r="AP74" s="7"/>
-      <c r="AQ74" s="7"/>
+      <c r="AN74" s="7">
+        <v>220.19</v>
+      </c>
+      <c r="AO74" s="7">
+        <v>82.22</v>
+      </c>
+      <c r="AP74" s="7">
+        <v>438</v>
+      </c>
+      <c r="AQ74" s="7">
+        <v>1899</v>
+      </c>
       <c r="AR74" s="41">
         <v>51.660000000000082</v>
       </c>
       <c r="AS74" s="41">
-        <f t="shared" si="82"/>
-        <v>-51.660000000000082</v>
+        <f t="shared" si="90"/>
+        <v>1847.34</v>
       </c>
       <c r="AT74" s="41">
         <f t="shared" ref="AT74:AT80" si="99">AN74-AN68</f>
-        <v>0</v>
+        <v>18.259999999999991</v>
       </c>
       <c r="AU74" s="41">
         <f t="shared" ref="AU74:AU80" si="100">AO74-AO68</f>
-        <v>0</v>
+        <v>12.469999999999999</v>
       </c>
       <c r="AV74" s="41">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AW74" s="26">
         <v>15</v>
@@ -17123,31 +18012,31 @@
       <c r="BD74" s="5"/>
       <c r="BE74" s="23"/>
       <c r="BF74" s="12">
+        <f t="shared" si="82"/>
+        <v>1.0231353599999996E-2</v>
+      </c>
+      <c r="BG74" s="13">
         <f t="shared" si="83"/>
-        <v>0</v>
-      </c>
-      <c r="BG74" s="13">
+        <v>14.733149183999995</v>
+      </c>
+      <c r="BH74" s="13">
+        <f t="shared" si="95"/>
+        <v>1905.2799999999997</v>
+      </c>
+      <c r="BI74" s="14">
+        <f t="shared" si="87"/>
+        <v>0.11556831541820627</v>
+      </c>
+      <c r="BJ74" s="14">
+        <f t="shared" si="88"/>
+        <v>0.1295235294117647</v>
+      </c>
+      <c r="BK74" s="14">
         <f t="shared" si="84"/>
         <v>0</v>
       </c>
-      <c r="BH74" s="13">
-        <f t="shared" si="97"/>
-        <v>1520</v>
-      </c>
-      <c r="BI74" s="14" t="str">
-        <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ74" s="14" t="str">
+      <c r="BL74" s="14">
         <f t="shared" si="89"/>
-        <v/>
-      </c>
-      <c r="BK74" s="14">
-        <f t="shared" si="85"/>
-        <v>0</v>
-      </c>
-      <c r="BL74" s="14">
-        <f t="shared" si="90"/>
         <v>0</v>
       </c>
       <c r="BM74" s="48" t="str">
@@ -17155,28 +18044,28 @@
         <v/>
       </c>
       <c r="BN74" s="36" t="str">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v/>
       </c>
       <c r="BO74" s="14">
         <f t="shared" si="47"/>
-        <v>11.4</v>
+        <v>12.384319999999997</v>
       </c>
       <c r="BP74" s="52" t="str">
+        <f t="shared" si="97"/>
+        <v/>
+      </c>
+      <c r="BQ74" s="29">
         <f t="shared" si="93"/>
-        <v/>
-      </c>
-      <c r="BQ74" s="29">
+        <v>0</v>
+      </c>
+      <c r="BR74" s="38">
         <f t="shared" si="94"/>
         <v>0</v>
       </c>
-      <c r="BR74" s="38">
-        <f t="shared" si="95"/>
-        <v>0</v>
-      </c>
       <c r="BS74" s="31">
-        <f t="shared" si="87"/>
-        <v>11.4</v>
+        <f t="shared" si="86"/>
+        <v>12.384319999999997</v>
       </c>
     </row>
     <row r="75" spans="1:71" x14ac:dyDescent="0.3">
@@ -17243,20 +18132,20 @@
         <v>137.11999999999989</v>
       </c>
       <c r="AS75" s="40">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-137.11999999999989</v>
       </c>
       <c r="AT75" s="40">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-181.29</v>
       </c>
       <c r="AU75" s="40">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-73.31</v>
       </c>
       <c r="AV75" s="40">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>485</v>
       </c>
       <c r="AW75" s="24">
         <v>15</v>
@@ -17288,15 +18177,15 @@
         <v>0</v>
       </c>
       <c r="BH75" s="9">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI75" s="10" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ75" s="10" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ75" s="10" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK75" s="10">
@@ -17304,7 +18193,7 @@
         <v>0</v>
       </c>
       <c r="BL75" s="10" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM75" s="10">
@@ -17320,7 +18209,7 @@
         <v/>
       </c>
       <c r="BP75" s="50">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v>0</v>
       </c>
       <c r="BQ75" s="27">
@@ -17399,20 +18288,20 @@
         <v>45.769999999999982</v>
       </c>
       <c r="AS76" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-45.769999999999982</v>
       </c>
       <c r="AT76" s="45">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-205.53</v>
       </c>
       <c r="AU76" s="45">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-79.069999999999993</v>
       </c>
       <c r="AV76" s="45">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>458</v>
       </c>
       <c r="AW76" s="25">
         <v>15</v>
@@ -17444,15 +18333,15 @@
         <v>0</v>
       </c>
       <c r="BH76" s="46">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI76" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ76" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ76" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK76" s="47">
@@ -17460,7 +18349,7 @@
         <v>0</v>
       </c>
       <c r="BL76" s="47" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM76" s="47">
@@ -17476,7 +18365,7 @@
         <v/>
       </c>
       <c r="BP76" s="51">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v>0</v>
       </c>
       <c r="BQ76" s="28">
@@ -17555,20 +18444,20 @@
         <v>84.700000000000045</v>
       </c>
       <c r="AS77" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-84.700000000000045</v>
       </c>
       <c r="AT77" s="45">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-287.8</v>
       </c>
       <c r="AU77" s="45">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-88.58</v>
       </c>
       <c r="AV77" s="45">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>338</v>
       </c>
       <c r="AW77" s="25">
         <v>15</v>
@@ -17600,15 +18489,15 @@
         <v>0</v>
       </c>
       <c r="BH77" s="46">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI77" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ77" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ77" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK77" s="47">
@@ -17616,7 +18505,7 @@
         <v>0</v>
       </c>
       <c r="BL77" s="47" t="str">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BM77" s="47">
@@ -17632,7 +18521,7 @@
         <v/>
       </c>
       <c r="BP77" s="51">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v>0</v>
       </c>
       <c r="BQ77" s="28">
@@ -17711,20 +18600,20 @@
         <v>47.420000000000073</v>
       </c>
       <c r="AS78" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-47.420000000000073</v>
       </c>
       <c r="AT78" s="45">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-273.05</v>
       </c>
       <c r="AU78" s="45">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-79.709999999999994</v>
       </c>
       <c r="AV78" s="45">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>362</v>
       </c>
       <c r="AW78" s="25">
         <v>15</v>
@@ -17755,15 +18644,15 @@
         <v>0</v>
       </c>
       <c r="BH78" s="46">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI78" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ78" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ78" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK78" s="47">
@@ -17771,7 +18660,7 @@
         <v>0</v>
       </c>
       <c r="BL78" s="47">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM78" s="48" t="str">
@@ -17787,7 +18676,7 @@
         <v>11.2875</v>
       </c>
       <c r="BP78" s="51" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v/>
       </c>
       <c r="BQ78" s="28">
@@ -17866,20 +18755,20 @@
         <v>133.55999999999995</v>
       </c>
       <c r="AS79" s="45">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-133.55999999999995</v>
       </c>
       <c r="AT79" s="45">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-310.07</v>
       </c>
       <c r="AU79" s="45">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-94.46</v>
       </c>
       <c r="AV79" s="45">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>295</v>
       </c>
       <c r="AW79" s="25">
         <v>15</v>
@@ -17910,15 +18799,15 @@
         <v>0</v>
       </c>
       <c r="BH79" s="46">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI79" s="47" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ79" s="47" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ79" s="47" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK79" s="47">
@@ -17926,7 +18815,7 @@
         <v>0</v>
       </c>
       <c r="BL79" s="47">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM79" s="48" t="str">
@@ -17942,7 +18831,7 @@
         <v>11.2875</v>
       </c>
       <c r="BP79" s="51" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v/>
       </c>
       <c r="BQ79" s="28">
@@ -18022,20 +18911,20 @@
         <v>51.660000000000082</v>
       </c>
       <c r="AS80" s="41">
-        <f t="shared" si="82"/>
+        <f t="shared" si="90"/>
         <v>-51.660000000000082</v>
       </c>
       <c r="AT80" s="41">
         <f t="shared" si="99"/>
-        <v>0</v>
+        <v>-220.19</v>
       </c>
       <c r="AU80" s="41">
         <f t="shared" si="100"/>
-        <v>0</v>
+        <v>-82.22</v>
       </c>
       <c r="AV80" s="41">
         <f t="shared" si="98"/>
-        <v>0</v>
+        <v>438</v>
       </c>
       <c r="AW80" s="26">
         <v>15</v>
@@ -18067,15 +18956,15 @@
         <v>0</v>
       </c>
       <c r="BH80" s="13">
-        <f t="shared" si="97"/>
+        <f t="shared" si="95"/>
         <v>1505</v>
       </c>
       <c r="BI80" s="14" t="str">
+        <f t="shared" si="87"/>
+        <v/>
+      </c>
+      <c r="BJ80" s="14" t="str">
         <f t="shared" si="88"/>
-        <v/>
-      </c>
-      <c r="BJ80" s="14" t="str">
-        <f t="shared" si="89"/>
         <v/>
       </c>
       <c r="BK80" s="14">
@@ -18083,7 +18972,7 @@
         <v>0</v>
       </c>
       <c r="BL80" s="14">
-        <f t="shared" si="90"/>
+        <f t="shared" si="89"/>
         <v>0</v>
       </c>
       <c r="BM80" s="36" t="str">
@@ -18099,7 +18988,7 @@
         <v>11.2875</v>
       </c>
       <c r="BP80" s="52" t="str">
-        <f t="shared" si="93"/>
+        <f t="shared" si="97"/>
         <v/>
       </c>
       <c r="BQ80" s="29">
@@ -18165,6 +19054,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -18387,34 +19303,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -18431,29 +19345,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>